<commit_message>
P0-T01: journal et statut de la tâche
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 11:48 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 11:50 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -1941,7 +1941,7 @@
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr"/>
@@ -13169,7 +13169,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">

</xml_diff>

<commit_message>
P0-T02: Script de vérification de l'environnement
scripts/verifier-env.py : tableau OK/MANQUANT/OPTIONNEL, exit 1 si outil requis absent.
Test : exit 0 sur ce poste, exit 1 avec PG_BIN vers un dossier vide.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -561,8 +561,8 @@
 </file>
 
 <file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I18" headerRowCount="1">
-  <autoFilter ref="A4:I18"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I19" headerRowCount="1">
+  <autoFilter ref="A4:I19"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Code"/>
     <tableColumn id="2" name="Tâche"/>
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 11:50 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 11:51 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -1980,10 +1980,14 @@
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
-        </is>
-      </c>
-      <c r="I30" s="5" t="inlineStr"/>
+          <t>EN_COURS</t>
+        </is>
+      </c>
+      <c r="I30" s="5" t="inlineStr">
+        <is>
+          <t>H-015</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
@@ -13211,7 +13215,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
@@ -13225,7 +13229,11 @@
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr"/>
-      <c r="J9" s="5" t="inlineStr"/>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>H-015 (OUVERTE)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
@@ -14495,7 +14503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -15228,8 +15236,55 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>H-015</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>P0-T02</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>OUVERTE</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-16 11:51</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>Que faire si PG_BIN pointe vers un dossier sans binaires PostgreSQL ?</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>PG_BIN est exclusif dans verifier-env.py (pas de repli), sinon le cas test PG_BIN vide ne peut jamais sortir en 1 ici</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>pg-test.py retombe sur les chemins par défaut : comportement différent entre les deux scripts</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>en attente</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="C5:C18">
+  <conditionalFormatting sqref="C5:C19">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"NON_FAIT"</formula>
     </cfRule>

</xml_diff>

<commit_message>
P0-T02: journal et statut de la tâche
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -1980,7 +1980,7 @@
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="I30" s="5" t="inlineStr">
@@ -13215,7 +13215,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">

</xml_diff>

<commit_message>
P0-T03: Valider l'instance PostgreSQL de test et le schéma de référence
scripts/tester-schema.py : instance jetable, schéma 01+02, tests d'intégrité 03.
Test : 18/18 vérifications conformes, exit 0, .pgtest/ supprimé.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -561,8 +561,8 @@
 </file>
 
 <file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I19" headerRowCount="1">
-  <autoFilter ref="A4:I19"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I20" headerRowCount="1">
+  <autoFilter ref="A4:I20"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Code"/>
     <tableColumn id="2" name="Tâche"/>
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 11:51 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 11:52 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -2023,10 +2023,14 @@
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
-        </is>
-      </c>
-      <c r="I31" s="5" t="inlineStr"/>
+          <t>EN_COURS</t>
+        </is>
+      </c>
+      <c r="I31" s="5" t="inlineStr">
+        <is>
+          <t>H-016</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
@@ -13261,7 +13265,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
@@ -13275,7 +13279,11 @@
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr"/>
-      <c r="J10" s="5" t="inlineStr"/>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>H-016 (OUVERTE)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
@@ -14503,7 +14511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -15283,8 +15291,55 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>H-016</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>P0-T03</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>OUVERTE</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-16 11:52</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>database/03-tests-integrite.sql compte-t-il 13 blocs ERREUR + 5 OK comme l'indique la tâche ?</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>Il contient 12 ERREUR + 6 OK (total 18 conforme) ; la répartition 13+5 est une erreur de décompte, seul le total compte</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>Si faux, un bloc attendu ERREUR manquerait dans le fichier 03</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>en attente</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="C5:C19">
+  <conditionalFormatting sqref="C5:C20">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"NON_FAIT"</formula>
     </cfRule>

</xml_diff>

<commit_message>
P0-T03: journal et statut de la tâche
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 11:52 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 11:53 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -2023,7 +2023,7 @@
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="I31" s="5" t="inlineStr">
@@ -13265,7 +13265,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">

</xml_diff>

<commit_message>
P0-T04: Conventions de build .NET centralisées
global.json, Directory.Build.props, Directory.Packages.props (12 paquets), .editorconfig.
Test : dotnet 10.0.401, build console 0 avertissement, TreatWarningsAsErrors=true.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -561,8 +561,8 @@
 </file>
 
 <file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I20" headerRowCount="1">
-  <autoFilter ref="A4:I20"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I21" headerRowCount="1">
+  <autoFilter ref="A4:I21"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Code"/>
     <tableColumn id="2" name="Tâche"/>
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 11:53 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 11:55 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -2066,10 +2066,14 @@
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
-        </is>
-      </c>
-      <c r="I32" s="5" t="inlineStr"/>
+          <t>EN_COURS</t>
+        </is>
+      </c>
+      <c r="I32" s="5" t="inlineStr">
+        <is>
+          <t>H-017</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
@@ -13311,7 +13315,7 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
@@ -13325,7 +13329,11 @@
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr"/>
-      <c r="J11" s="5" t="inlineStr"/>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>H-017 (OUVERTE)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
@@ -14511,7 +14519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -15338,8 +15346,55 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>H-017</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>P0-T04</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>OUVERTE</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-16 11:55</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>FluentAssertions 8.x (licence commerciale Xceed) est-il acceptable pour un projet d'État ?</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>Version 8.11.0 retenue pour l'instant ; si la licence pose problème, épingler 7.x (Apache 2.0) dans Directory.Packages.props</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>Aucun avant l'écriture des premiers tests (P0-T05+ ou P1)</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>en attente</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="C5:C20">
+  <conditionalFormatting sqref="C5:C21">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"NON_FAIT"</formula>
     </cfRule>

</xml_diff>

<commit_message>
P0-T04: journal et statut de la tâche
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 11:55 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 11:56 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -2066,7 +2066,7 @@
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="I32" s="5" t="inlineStr">
@@ -13315,7 +13315,7 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">

</xml_diff>

<commit_message>
P0-T05: Modèles GitLab et guide de contribution
Modèle de MR de phase, modèles d'issue Anomalie/Demande, CONTRIBUTING.md (6 sections).
Test : 4 fichiers présents, grep -c '^## ' = 6.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -2109,7 +2109,7 @@
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="I33" s="5" t="inlineStr"/>
@@ -13361,7 +13361,7 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">

</xml_diff>

<commit_message>
P0-T05: journal et statut de la tâche
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 11:56 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 11:58 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -2109,7 +2109,7 @@
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="I33" s="5" t="inlineStr"/>
@@ -13361,7 +13361,7 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">

</xml_diff>

<commit_message>
P0-T06: Rapport d'outillage Claude Code
docs/OUTILLAGE.md : ponytail, ui-ux-pro-max, motion-design installés ; graphify manquant (H-018).
Test : 4 outils listés avec statut, backlog.py contexte exit 0.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -561,8 +561,8 @@
 </file>
 
 <file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I21" headerRowCount="1">
-  <autoFilter ref="A4:I21"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I22" headerRowCount="1">
+  <autoFilter ref="A4:I22"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Code"/>
     <tableColumn id="2" name="Tâche"/>
@@ -2148,12 +2148,12 @@
       </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="I34" s="5" t="inlineStr">
         <is>
-          <t>H-003</t>
+          <t>H-003, H-018</t>
         </is>
       </c>
     </row>
@@ -13403,7 +13403,7 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
@@ -13419,7 +13419,8 @@
       <c r="I13" s="5" t="inlineStr"/>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>H-003 (REPONDUE)</t>
+          <t>H-003 (REPONDUE)
+H-018 (OUVERTE)</t>
         </is>
       </c>
     </row>
@@ -14519,7 +14520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -15393,8 +15394,55 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>H-018</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>P0-T06</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>OUVERTE</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-16 11:58</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>graphify (CLI, paquet PyPI graphifyy) est absent du poste et uv (requis pour l'installer) est absent aussi : faut-il les installer maintenant pour le graphe de connaissances du code ?</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>Ne pas installer maintenant : graphify n'est utile qu'à partir de la première phase qui produit du code (P1). Installation prévue via scripts/installer-outils.ps1 (étapes uv puis uv tool install graphifyy, puis graphify install --project) avant P1 ; en attendant, la recherche se fait par Grep/Explore.</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>Sans graphify, les requêtes 'graphify query' de CLAUDE.md ne fonctionnent pas : le repérage du code se fait par recherche classique (plus lent, plus de tokens). Aucun blocage de P0.</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>en attente</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="C5:C21">
+  <conditionalFormatting sqref="C5:C22">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"NON_FAIT"</formula>
     </cfRule>

</xml_diff>

<commit_message>
P0-T06: journal et statut de la tâche
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 11:58 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 12:00 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -1083,7 +1083,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -2148,7 +2148,7 @@
       </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="I34" s="5" t="inlineStr">
@@ -13069,7 +13069,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
     </row>
@@ -13403,7 +13403,7 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">

</xml_diff>

<commit_message>
P0: clôture de phase
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 12:00 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 12:21 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -1083,7 +1083,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDEE</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -1941,7 +1941,7 @@
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr"/>
@@ -1980,7 +1980,7 @@
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="I30" s="5" t="inlineStr">
@@ -2023,7 +2023,7 @@
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="I31" s="5" t="inlineStr">
@@ -2066,7 +2066,7 @@
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="I32" s="5" t="inlineStr">
@@ -2109,7 +2109,7 @@
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="I33" s="5" t="inlineStr"/>
@@ -2148,7 +2148,7 @@
       </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="I34" s="5" t="inlineStr">
@@ -13069,7 +13069,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDEE</t>
         </is>
       </c>
     </row>
@@ -13181,7 +13181,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
@@ -13223,7 +13223,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
@@ -13269,7 +13269,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
@@ -13315,7 +13315,7 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
@@ -13361,7 +13361,7 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
@@ -13403,7 +13403,7 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Adaptation : dépôt GitHub et CI GitHub Actions
- P3 : workflow GitHub Actions (.github/workflows/ci.yml), image sur ghcr.io,
  modèles de pull request GitHub (au lieu de .gitlab-ci.yml)
- CLAUDE.md, DEMARRAGE.md, valider-phase, garde.py : push vers GitHub,
  dépôt public = rien de sensible
- H-002 répondue (choix utilisateur) ; GitLab reste une intégration
  fonctionnelle de la plateforme (P12-P13)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 12:21 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 12:48 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -1192,7 +1192,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Conteneurisation et intégration continue GitLab</t>
+          <t>Conteneurisation et intégration continue GitHub Actions</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -2951,7 +2951,7 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>P3 · Conteneurisation et intégration continue GitLab</t>
+          <t>P3 · Conteneurisation et intégration continue GitHub Actions</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
@@ -2994,7 +2994,7 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>P3 · Conteneurisation et intégration continue GitLab</t>
+          <t>P3 · Conteneurisation et intégration continue GitHub Actions</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
@@ -3033,7 +3033,7 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>P3 · Conteneurisation et intégration continue GitLab</t>
+          <t>P3 · Conteneurisation et intégration continue GitHub Actions</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
@@ -3072,7 +3072,7 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>P3 · Conteneurisation et intégration continue GitLab</t>
+          <t>P3 · Conteneurisation et intégration continue GitHub Actions</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
@@ -3082,7 +3082,7 @@
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>Pipeline .gitlab-ci.yml</t>
+          <t>Workflow GitHub Actions</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
@@ -3115,7 +3115,7 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>P3 · Conteneurisation et intégration continue GitLab</t>
+          <t>P3 · Conteneurisation et intégration continue GitHub Actions</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
@@ -14655,7 +14655,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>OUVERTE</t>
+          <t>REPONDUE</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -14685,7 +14685,7 @@
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>en attente</t>
+          <t>48) : Choix utilisateur (2026-10-16) : le dépôt du projet est sur GitHub (hajar-hamid-coder/gprojet, public) ; l'intégration continue se fait avec GitHub Actions et l'image est publiée sur ghcr.io. GitLab reste une intégration fonctionnelle de la plateforme (P12-P13).</t>
         </is>
       </c>
     </row>
@@ -17115,14 +17115,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>P3 · Conteneurisation et intégration continue GitLab</t>
+          <t>P3 · Conteneurisation et intégration continue GitHub Actions</t>
         </is>
       </c>
     </row>
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>Objectif : images Docker, environnement local complet par docker compose, pipeline GitLab CI. Livrable : docker compose up fonctionnel et .gitlab-ci.yml. ⚠️ Nécessite Docker (hypothèse H-001).</t>
+          <t>Objectif : images Docker, environnement local complet par docker compose, intégration continue GitHub Actions sur le dépôt hajar-hamid-coder/gprojet. Livrable : docker compose up fonctionnel et .github/workflows/ci.yml. ⚠️ Nécessite Docker (hypothèse H-001).</t>
         </is>
       </c>
     </row>
@@ -17361,7 +17361,7 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Pipeline .gitlab-ci.yml</t>
+          <t>Workflow GitHub Actions</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -17381,18 +17381,18 @@
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>étapes build, test (service postgres:18, rapports JUnit et couverture Cobertura), qualite (dotnet format --verify-no-changes), securite (templates GitLab SAST, Dependency-Scanning, Secret-Detection, Container-Scanning), paquet (build et push des images vers le GitLab Container Registry sur main et les tags), deploiement (manuel, préparé pour P13). Cache NuGet.</t>
+          <t>.github/workflows/ci.yml déclenché sur push et pull request : jobs build, test (service postgres:18, GP_TEST_CONNECTION, rapport de tests et couverture publiés comme artefacts), qualite (dotnet format --verify-no-changes), securite (CodeQL C#, dependency-review sur les pull requests, scan d'image Trivy), paquet (build et push de l'image vers GitHub Container Registry ghcr.io sur main et les tags, avec GITHUB_TOKEN), deploiement (workflow_dispatch + environnement protégé, préparé pour P13). Cache NuGet, versions d'actions épinglées. Reprendre aussi les modèles .gitlab/ existants en .github/pull_request_template.md et .github/ISSUE_TEMPLATE/, et mettre CONTRIBUTING.md à jour (pull requests GitHub).</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>python scripts/verifier-ci.py (à écrire, parse YAML) confirme les 6 étapes, les rapports JUnit, l'absence de secret en clair ; validation par l'API CI Lint de GitLab si H-002 est répondue, sinon signalée dans la preuve.</t>
+          <t>python scripts/verifier-ci.py (à écrire, parse YAML) confirme les 6 jobs, leurs dépendances, le service PostgreSQL et l'absence de secret en clair ; le modèle de pull request existe. L'exécution réelle sur GitHub se constate après le push de l'utilisateur (signalé dans le bilan de phase).</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr"/>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>H-002 (OUVERTE)</t>
+          <t>H-002 (REPONDUE)</t>
         </is>
       </c>
     </row>
@@ -17427,7 +17427,7 @@
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>docs/DEPLOIEMENT.md : prérequis, variables, démarrage compose, migrations, dépannage, description du pipeline et des variables CI à créer dans GitLab (masquées / protégées).</t>
+          <t>docs/DEPLOIEMENT.md : prérequis, variables, démarrage compose, migrations, dépannage, description du workflow GitHub Actions, des secrets à créer (Settings → Secrets and variables → Actions) et de la publication d'image sur ghcr.io.</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">

</xml_diff>

<commit_message>
P0: note de demande pour P1 (FluentAssertions 7.x, migration .github)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 12:48 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 12:51 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -13331,7 +13331,7 @@
       <c r="I11" s="5" t="inlineStr"/>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>H-017 (OUVERTE)</t>
+          <t>H-017 (REPONDUE)</t>
         </is>
       </c>
     </row>
@@ -15360,7 +15360,7 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>OUVERTE</t>
+          <t>REPONDUE</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
@@ -15390,7 +15390,7 @@
       </c>
       <c r="I21" s="5" t="inlineStr">
         <is>
-          <t>en attente</t>
+          <t>51) : Non : épingler FluentAssertions 7.x (Apache 2.0), pas de licence commerciale</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
backlog : demandes utilisateur visibles dans P1-T01
- backlog.py voir affiche désormais les notes du journal de la tâche
- P1-T01 : FluentAssertions 7.x (H-017) et migration .gitlab/ -> .github/
- P3-T04 : vérifie les modèles .github/ au lieu de les créer

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 12:51 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 12:53 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -15957,12 +15957,12 @@
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Gprojet.slnx ; un seul projet backend src/Gprojet-Backend/Gprojet-Backend.csproj (Microsoft.NET.Sdk.Web, RootNamespace Gprojet.Backend) avec les dossiers-couches Web/, Orchestration/, Services/, Mapping/, Repositories/, Entities/, Contracts/, Infrastructure/, Common/ (espaces de noms alignés sur les dossiers) ; projet de tests tests/Gprojet-Backend.Tests (xUnit) avec Unitaires/, Integration/, Architecture/. Aucun autre projet (le front arrive en P2-T01).</t>
+          <t>Gprojet.slnx ; un seul projet backend src/Gprojet-Backend/Gprojet-Backend.csproj (Microsoft.NET.Sdk.Web, RootNamespace Gprojet.Backend) avec les dossiers-couches Web/, Orchestration/, Services/, Mapping/, Repositories/, Entities/, Contracts/, Infrastructure/, Common/ (espaces de noms alignés sur les dossiers) ; projet de tests tests/Gprojet-Backend.Tests (xUnit) avec Unitaires/, Integration/, Architecture/. Aucun autre projet (le front arrive en P2-T01). Demandes utilisateur à intégrer dans cette tâche : Directory.Packages.props → FluentAssertions en dernière 7.x stable (licence Apache 2.0, H-017) au lieu de 8.x ; migrer .gitlab/ vers .github/ (pull_request_template.md, ISSUE_TEMPLATE/Anomalie.md et Demande.md) et adapter CONTRIBUTING.md (pull requests GitHub).</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>dotnet build Gprojet.slnx réussit sans avertissement ; dotnet sln Gprojet.slnx list affiche exactement 2 projets (Gprojet-Backend, Gprojet-Backend.Tests) ; dotnet test passe (test de fumée).</t>
+          <t>dotnet build Gprojet.slnx réussit sans avertissement ; dotnet sln Gprojet.slnx list affiche exactement 2 projets (Gprojet-Backend, Gprojet-Backend.Tests) ; dotnet test passe (test de fumée). Directory.Packages.props référence FluentAssertions 7.x ; .gitlab/ n'existe plus et .github/pull_request_template.md existe.</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr"/>
@@ -17381,12 +17381,12 @@
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>.github/workflows/ci.yml déclenché sur push et pull request : jobs build, test (service postgres:18, GP_TEST_CONNECTION, rapport de tests et couverture publiés comme artefacts), qualite (dotnet format --verify-no-changes), securite (CodeQL C#, dependency-review sur les pull requests, scan d'image Trivy), paquet (build et push de l'image vers GitHub Container Registry ghcr.io sur main et les tags, avec GITHUB_TOKEN), deploiement (workflow_dispatch + environnement protégé, préparé pour P13). Cache NuGet, versions d'actions épinglées. Reprendre aussi les modèles .gitlab/ existants en .github/pull_request_template.md et .github/ISSUE_TEMPLATE/, et mettre CONTRIBUTING.md à jour (pull requests GitHub).</t>
+          <t>.github/workflows/ci.yml déclenché sur push et pull request : jobs build, test (service postgres:18, GP_TEST_CONNECTION, rapport de tests et couverture publiés comme artefacts), qualite (dotnet format --verify-no-changes), securite (CodeQL C#, dependency-review sur les pull requests, scan d'image Trivy), paquet (build et push de l'image vers GitHub Container Registry ghcr.io sur main et les tags, avec GITHUB_TOKEN), deploiement (workflow_dispatch + environnement protégé, préparé pour P13). Cache NuGet, versions d'actions épinglées. Vérifier que les modèles .github/ (faits en P1-T01) sont cohérents avec le workflow.</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>python scripts/verifier-ci.py (à écrire, parse YAML) confirme les 6 jobs, leurs dépendances, le service PostgreSQL et l'absence de secret en clair ; le modèle de pull request existe. L'exécution réelle sur GitHub se constate après le push de l'utilisateur (signalé dans le bilan de phase).</t>
+          <t>python scripts/verifier-ci.py (à écrire, parse YAML) confirme les 6 jobs, leurs dépendances, le service PostgreSQL et l'absence de secret en clair ; les modèles .github/ sont présents. L'exécution réelle sur GitHub se constate après le push de l'utilisateur (signalé dans le bilan de phase).</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
P1-T01: Créer la solution et le projet Gprojet-Backend
Gprojet.slnx, src/Gprojet-Backend (dossiers-couches), tests/Gprojet-Backend.Tests (test de fumée).
Demandes utilisateur : FluentAssertions 7.2.2 (Apache 2.0, H-017) ; modèles .gitlab/ migrés vers .github/
et CONTRIBUTING.md adapté à GitHub (pull requests, GitHub Actions).
Test : build 0 avertissement, 2 projets, dotnet test 1/1.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 12:53 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 12:54 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1121,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>NON_DEMARREE</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -2191,7 +2191,7 @@
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="I35" s="5" t="inlineStr"/>
@@ -15840,7 +15840,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>NON_DEMARREE</t>
+          <t>EN_COURS</t>
         </is>
       </c>
     </row>
@@ -15952,7 +15952,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">

</xml_diff>

<commit_message>
P1-T01: journal et statut de la tâche
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 12:54 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 12:57 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -2191,7 +2191,7 @@
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="I35" s="5" t="inlineStr"/>
@@ -15952,7 +15952,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">

</xml_diff>

<commit_message>
P1-T02: Tests d'architecture par espace de noms
12 règles NetArchTest entre couches Gprojet.Backend.*, chacune avec un garde-fou
(violations simulées dans le projet de test, échecs attendus exacts) + test de couverture.
Test : --filter Category=Architecture → 25/25 ; dotnet test → 26/26 ; build 0 avertissement.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -561,8 +561,8 @@
 </file>
 
 <file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I22" headerRowCount="1">
-  <autoFilter ref="A4:I22"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I23" headerRowCount="1">
+  <autoFilter ref="A4:I23"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Code"/>
     <tableColumn id="2" name="Tâche"/>
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 12:57 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 13:01 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -2230,10 +2230,14 @@
       </c>
       <c r="H36" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
-        </is>
-      </c>
-      <c r="I36" s="5" t="inlineStr"/>
+          <t>EN_COURS</t>
+        </is>
+      </c>
+      <c r="I36" s="5" t="inlineStr">
+        <is>
+          <t>H-019</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="n">
@@ -14520,7 +14524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -15441,8 +15445,55 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>H-019</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>P1-T02</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>OUVERTE</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-16 13:01</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>Comment reconnaître un contrôleur, et la liste blanche System.* de Contracts suffit-elle ?</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>Contrôleur = hérite de ControllerBase ou nom en *Controller ; Contracts autorise tout System.* (les API absentes du navigateur ne sont pas détectées, la compilation du front en P2 servira de seconde garde)</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>Des endpoints minimal API échapperaient à la règle ; une API System non disponible en WASM serait détectée seulement à la compilation du front</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="inlineStr">
+        <is>
+          <t>en attente</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="C5:C22">
+  <conditionalFormatting sqref="C5:C23">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"NON_FAIT"</formula>
     </cfRule>
@@ -15994,7 +16045,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
@@ -16008,7 +16059,11 @@
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr"/>
-      <c r="J9" s="5" t="inlineStr"/>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>H-019 (OUVERTE)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">

</xml_diff>

<commit_message>
P1-T02: journal et statut de la tâche
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 13:01 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 13:02 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -2230,7 +2230,7 @@
       </c>
       <c r="H36" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="I36" s="5" t="inlineStr">
@@ -16045,7 +16045,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">

</xml_diff>

<commit_message>
P1-T03: Common : primitives transverses
Result/Result<T>, 4 exceptions métier, PageRequete/PageResultat (taille max 200, bornage),
ICurrentUser, IHorloge + HorlogeSysteme (Aujourdhui en Africa/Casablanca, H-020), IGenerateurCode.
Test : --filter Category=Common → 16/16 ; dotnet test → 42/42 ; build 0 avertissement.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -561,8 +561,8 @@
 </file>
 
 <file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I23" headerRowCount="1">
-  <autoFilter ref="A4:I23"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I24" headerRowCount="1">
+  <autoFilter ref="A4:I24"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Code"/>
     <tableColumn id="2" name="Tâche"/>
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 13:02 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 13:05 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -2273,10 +2273,14 @@
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
-        </is>
-      </c>
-      <c r="I37" s="5" t="inlineStr"/>
+          <t>EN_COURS</t>
+        </is>
+      </c>
+      <c r="I37" s="5" t="inlineStr">
+        <is>
+          <t>H-020</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="n">
@@ -14524,7 +14528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -15492,8 +15496,55 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>H-020</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>P1-T03</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>OUVERTE</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-16 13:05</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>Dans quel fuseau calcule-t-on la date du jour (saisie des temps, échéances) ?</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>Fuseau Africa/Casablanca (HCP) ; IHorloge.Aujourdhui est calculé dans ce fuseau, Maintenant reste en UTC</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>Si un autre fuseau est attendu, changer la valeur passée à HorlogeSysteme ; en UTC pur, les saisies entre minuit et 1 h seraient datées de la veille</t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t>en attente</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="C5:C23">
+  <conditionalFormatting sqref="C5:C24">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"NON_FAIT"</formula>
     </cfRule>
@@ -16091,7 +16142,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
@@ -16105,7 +16156,11 @@
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr"/>
-      <c r="J10" s="5" t="inlineStr"/>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>H-020 (OUVERTE)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">

</xml_diff>

<commit_message>
P1-T03: journal et statut de la tâche
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 13:05 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 13:08 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -2273,7 +2273,7 @@
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="I37" s="5" t="inlineStr">
@@ -16142,7 +16142,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">

</xml_diff>

<commit_message>
P1-T04: journal et statut de la tâche
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 13:15 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 13:16 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -2316,7 +2316,7 @@
       </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="I38" s="5" t="inlineStr">
@@ -16239,7 +16239,7 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">

</xml_diff>

<commit_message>
P1-T04: Entités du domaine (6 schémas)
EntiteAuditable (uuid v7, audit, suppression logique, VersionLigne/xmin), 60 entités POCO
par module, 49 énumérations, Common/ValeurEnumSql (enum ⇄ texte SQL), Historique en bigint.
Test : --filter Category=Entites → 57/57 (60 types = 60 tables, enums = CHECK IN) ; dotnet test → 99/99.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -561,8 +561,8 @@
 </file>
 
 <file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I24" headerRowCount="1">
-  <autoFilter ref="A4:I24"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I25" headerRowCount="1">
+  <autoFilter ref="A4:I25"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Code"/>
     <tableColumn id="2" name="Tâche"/>
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 13:08 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 13:15 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -2316,10 +2316,14 @@
       </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
-        </is>
-      </c>
-      <c r="I38" s="5" t="inlineStr"/>
+          <t>EN_COURS</t>
+        </is>
+      </c>
+      <c r="I38" s="5" t="inlineStr">
+        <is>
+          <t>H-021</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="n">
@@ -14528,7 +14532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -15543,8 +15547,55 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>H-021</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>P1-T04</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>OUVERTE</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-16 13:15</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>patte.card_min (CHECK IN numérique 0,1) et correspondance_type.type_logique (sans CHECK) doivent-ils devenir des énumérations ?</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>Non : card_min reste short, correspondance_type.type_logique reste string ; seuls les CHECK IN à valeurs texte deviennent des enums (49 enums, 54 contraintes contrôlées)</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>Si faux : créer CardinaliteMin et/ou ajouter le CHECK au SQL puis typer en TypeLogique</t>
+        </is>
+      </c>
+      <c r="I25" s="5" t="inlineStr">
+        <is>
+          <t>en attente</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="C5:C24">
+  <conditionalFormatting sqref="C5:C25">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"NON_FAIT"</formula>
     </cfRule>
@@ -16188,7 +16239,7 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
@@ -16202,7 +16253,11 @@
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr"/>
-      <c r="J11" s="5" t="inlineStr"/>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>H-021 (OUVERTE)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">

</xml_diff>

<commit_message>
P1-T05: DbContext et configurations EF Core
GpDbContext (Repositories/, extension ltree, snake_case maison, convertisseur enum unique,
filtre !EstSupprime, xmin), 60 IEntityTypeConfiguration fidèles à 01-schema.sql
(CHECK, index uniques partiels, GiST, criticite générée), fabrique design-time
lisant ConnectionStrings__Gp, dotnet-ef 10.0.13 en outil local.
Test : dbcontext info OK ; --filter Category=Persistance → 5/5 ; dotnet test → 104/104.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -561,8 +561,8 @@
 </file>
 
 <file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I25" headerRowCount="1">
-  <autoFilter ref="A4:I25"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I26" headerRowCount="1">
+  <autoFilter ref="A4:I26"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Code"/>
     <tableColumn id="2" name="Tâche"/>
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 13:16 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 13:27 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -2359,10 +2359,14 @@
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
-        </is>
-      </c>
-      <c r="I39" s="5" t="inlineStr"/>
+          <t>EN_COURS</t>
+        </is>
+      </c>
+      <c r="I39" s="5" t="inlineStr">
+        <is>
+          <t>H-022</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="n">
@@ -14532,7 +14536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -15594,8 +15598,55 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>H-022</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>P1-T05</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>OUVERTE</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-16 13:27</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>Comment reproduire l'index sur expression ux_agent_email (lower(email)) et le trigger de lecture seule de commun.historique, non modélisables par EF ?</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>Le modèle EF déclare ux_agent_email sur email (shortcut commenté) ; la migration initiale P1-T06 recrée l'index sur lower(email) et le trigger tg_historique_lecture_seule en SQL brut</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>Si oublié en P1-T06 : unicité de l'email sensible à la casse et journal d'historique modifiable</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>en attente</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="C5:C25">
+  <conditionalFormatting sqref="C5:C26">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"NON_FAIT"</formula>
     </cfRule>
@@ -16285,7 +16336,7 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
@@ -16299,7 +16350,11 @@
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr"/>
-      <c r="J12" s="5" t="inlineStr"/>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>H-022 (OUVERTE)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">

</xml_diff>

<commit_message>
P1-T05: journal et statut de la tâche
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 13:27 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 14:32 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -2359,7 +2359,7 @@
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="I39" s="5" t="inlineStr">
@@ -16336,7 +16336,7 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">

</xml_diff>

<commit_message>
P1-T06: Migration initiale identique au schéma de référence
InitialCreate (ux_agent_email sur lower(email) et trigger d'ajout seul de commun.historique
en SQL brut, données de référence en ressource embarquée), scripts/comparer-schema.py
(01-schema.sql vs migration sur l'instance jetable, pg_catalog, bidirectionnel, --auto-test).
Migration appliquée à gprojet.
Test : comparer-schema → 0 écart ; --auto-test → 3/3 ; gprojet 60 tables / 6 schémas ; dotnet test → 104/104.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -561,8 +561,8 @@
 </file>
 
 <file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I26" headerRowCount="1">
-  <autoFilter ref="A4:I26"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I27" headerRowCount="1">
+  <autoFilter ref="A4:I27"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Code"/>
     <tableColumn id="2" name="Tâche"/>
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 14:32 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 14:45 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -2402,10 +2402,14 @@
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
-        </is>
-      </c>
-      <c r="I40" s="5" t="inlineStr"/>
+          <t>EN_COURS</t>
+        </is>
+      </c>
+      <c r="I40" s="5" t="inlineStr">
+        <is>
+          <t>H-023</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="n">
@@ -14536,7 +14540,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -15645,8 +15649,55 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>H-023</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>P1-T06</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>OUVERTE</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-16 14:45</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>La comparaison de schéma doit-elle couvrir l'ordre des colonnes et le contenu des données de référence ?</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>Non : type, nullabilité, défaut, contraintes, index, triggers, fonctions et nombre de lignes par table suffisent ; les données sont une copie figée de 02 embarquée dans la migration</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>Une différence d'ordre de colonnes ou de valeurs (même nombre de lignes) ne serait pas détectée</t>
+        </is>
+      </c>
+      <c r="I27" s="5" t="inlineStr">
+        <is>
+          <t>en attente</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="C5:C26">
+  <conditionalFormatting sqref="C5:C27">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"NON_FAIT"</formula>
     </cfRule>
@@ -16382,7 +16433,7 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
@@ -16396,7 +16447,11 @@
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr"/>
-      <c r="J13" s="5" t="inlineStr"/>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>H-023 (OUVERTE)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">

</xml_diff>

<commit_message>
P1-T06: journal et statut de la tâche
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -2402,7 +2402,7 @@
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="I40" s="5" t="inlineStr">
@@ -16433,7 +16433,7 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">

</xml_diff>

<commit_message>
P1-T07: Intercepteurs : audit, suppression logique, historique chaîné
AuditInterceptor (cree_*/modifie_* via ICurrentUser/IHorloge, Remove → suppression logique,
historique par champ chaîné en sha256 sous pg_advisory_xact_lock dans la même transaction),
EmpreinteHistorique (sérialisation canonique), VerificateurChaineHistorique, ContexteRequete.
Test : --filter Category=Integration → 7/7 (audit, suppression, chaîne, altération SQL détectée,
concurrence, rollback) ; dotnet test → 111/111.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -561,8 +561,8 @@
 </file>
 
 <file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I27" headerRowCount="1">
-  <autoFilter ref="A4:I27"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I28" headerRowCount="1">
+  <autoFilter ref="A4:I28"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Code"/>
     <tableColumn id="2" name="Tâche"/>
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 14:45 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 14:49 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -2445,10 +2445,14 @@
       </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
-        </is>
-      </c>
-      <c r="I41" s="5" t="inlineStr"/>
+          <t>EN_COURS</t>
+        </is>
+      </c>
+      <c r="I41" s="5" t="inlineStr">
+        <is>
+          <t>H-024</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="n">
@@ -14540,7 +14544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -15696,8 +15700,55 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>H-024</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>P1-T07</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>OUVERTE</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-16 14:49</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>Quel agent pour les écritures hors requête (jobs, données initiales), et type_cible sans schéma est-il acceptable ?</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>Un utilisateur système (ICurrentUser dédié) sera fourni pour les traitements hors requête ; type_cible = nom de table sans schéma (unique entre schémas, ≤ 30 caractères)</t>
+        </is>
+      </c>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>Sans utilisateur système, cree_par/agent_id seraient vides pour ces écritures ; un futur doublon de nom de table entre schémas rendrait type_cible ambigu</t>
+        </is>
+      </c>
+      <c r="I28" s="5" t="inlineStr">
+        <is>
+          <t>en attente</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="C5:C27">
+  <conditionalFormatting sqref="C5:C28">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"NON_FAIT"</formula>
     </cfRule>
@@ -16479,7 +16530,7 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -16493,7 +16544,11 @@
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr"/>
-      <c r="J14" s="5" t="inlineStr"/>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>H-024 (OUVERTE)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">

</xml_diff>

<commit_message>
P1-T07: journal et statut de la tâche
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 14:49 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 14:51 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -2445,7 +2445,7 @@
       </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="I41" s="5" t="inlineStr">
@@ -16530,7 +16530,7 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">

</xml_diff>

<commit_message>
P1-T08: Unit of Work et repositories de base
IUnitOfWork/UnitOfWork (CommitAsync : concurrence xmin → ConflitException ; transaction explicite
réentrante compatible avec l'AuditInterceptor), RepositoryBase<T> interne (GetById, Ajouter,
Supprimer logique, pagination déterministe), premier agrégat ICompetenceRepository.
Test : --filter Category=Integration → 12/12 (atomicité, concurrence) ; dotnet test → 116/116.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -561,8 +561,8 @@
 </file>
 
 <file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I28" headerRowCount="1">
-  <autoFilter ref="A4:I28"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I29" headerRowCount="1">
+  <autoFilter ref="A4:I29"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Code"/>
     <tableColumn id="2" name="Tâche"/>
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 14:51 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 14:54 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -2488,10 +2488,14 @@
       </c>
       <c r="H42" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
-        </is>
-      </c>
-      <c r="I42" s="5" t="inlineStr"/>
+          <t>EN_COURS</t>
+        </is>
+      </c>
+      <c r="I42" s="5" t="inlineStr">
+        <is>
+          <t>H-025</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="n">
@@ -14544,7 +14548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -15747,8 +15751,55 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>H-025</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>P1-T08</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>OUVERTE</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-16 14:54</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>Quels repositories d'agrégat livrer dans le socle, et où enregistrer UnitOfWork/repositories dans la DI ?</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>Un seul repository réel (Compétence) pour démontrer le motif ; les autres arrivent avec leurs modules (P4, P5…). Enregistrement DI dans la tâche de composition (P1-T09/T10)</t>
+        </is>
+      </c>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>Effort minime pour changer d'agrégat ; aucun enregistrement DI tant que Program.cs n'est pas composé</t>
+        </is>
+      </c>
+      <c r="I29" s="5" t="inlineStr">
+        <is>
+          <t>en attente</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="C5:C28">
+  <conditionalFormatting sqref="C5:C29">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"NON_FAIT"</formula>
     </cfRule>
@@ -16576,7 +16627,7 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
@@ -16590,7 +16641,11 @@
         </is>
       </c>
       <c r="I15" s="5" t="inlineStr"/>
-      <c r="J15" s="5" t="inlineStr"/>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>H-025 (OUVERTE)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">

</xml_diff>

<commit_message>
P1-T08: journal et statut de la tâche
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 14:54 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 14:55 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -2488,7 +2488,7 @@
       </c>
       <c r="H42" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="I42" s="5" t="inlineStr">
@@ -16627,7 +16627,7 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">

</xml_diff>

<commit_message>
P1-T09: Socle API : DI, erreurs, OpenAPI, logs, santé
Program.cs minimal, AddGpRepositories/AddGpInfrastructure/AddGpWeb, IExceptionHandler →
ProblemDetails (400/403/404/409/422/500, détail seulement en Development), OpenAPI natif +
Scalar (Development, ressources locales), Serilog JSON, /health et /health/ready (base),
ICurrentUser provisoire SYSTEME (shortcut jusqu'à P18).
Test : dotnet test → 124/124 (WebApplicationFactory sur pg-test) ; dotnet run → /health/ready 200 sur gprojet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -561,8 +561,8 @@
 </file>
 
 <file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I29" headerRowCount="1">
-  <autoFilter ref="A4:I29"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I30" headerRowCount="1">
+  <autoFilter ref="A4:I30"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Code"/>
     <tableColumn id="2" name="Tâche"/>
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 14:55 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 15:00 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -2531,12 +2531,12 @@
       </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="I43" s="5" t="inlineStr">
         <is>
-          <t>H-004</t>
+          <t>H-004, H-026</t>
         </is>
       </c>
     </row>
@@ -14548,7 +14548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -15798,8 +15798,55 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>H-026</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>P1-T09</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>OUVERTE</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-16 15:00</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>Quel utilisateur courant avant Keycloak (P18), et quel code HTTP pour RegleMetierException ?</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>ICurrentUser provisoire = agent SYSTEME (Id Guid.Empty, sans rôle), shortcut à remplacer en P18 ; RegleMetierException → 422, validation FluentValidation → 400</t>
+        </is>
+      </c>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>cree_par/agent_id valent Guid.Empty jusqu'en P18 (colonnes sans FK) ; changer le code 422 est une ligne dans GestionnaireExceptions</t>
+        </is>
+      </c>
+      <c r="I30" s="5" t="inlineStr">
+        <is>
+          <t>en attente</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="C5:C29">
+  <conditionalFormatting sqref="C5:C30">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"NON_FAIT"</formula>
     </cfRule>
@@ -16673,7 +16720,7 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
@@ -16689,7 +16736,8 @@
       <c r="I16" s="5" t="inlineStr"/>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>H-004 (REPONDUE)</t>
+          <t>H-004 (REPONDUE)
+H-026 (OUVERTE)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
P1-T09: journal et statut de la tâche
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -2531,7 +2531,7 @@
       </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="I43" s="5" t="inlineStr">
@@ -16720,7 +16720,7 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">

</xml_diff>

<commit_message>
P1-T10: journal et statut de la tâche
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 15:11 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 15:14 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -2574,7 +2574,7 @@
       </c>
       <c r="H44" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="I44" s="5" t="inlineStr">
@@ -16818,7 +16818,7 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">

</xml_diff>

<commit_message>
P1-T10: Authentification de développement et utilisateur courant
DevAuthHandler (schéma Dev, en-tête X-Dev-Matricule, uniquement Development/Test), schéma Refus
ailleurs (401), rôles déduits RESPONSABLE_ENTITE / DELEGATAIRE, UtilisateurCourant (claims, repli
SYSTEME hors requête), contrôleurs authentifiés par défaut.
Test : AuthDevTests 11/11 (401 sans en-tête/inconnu/inactif/supprimé, 200 + ICurrentUser, Production
sans schéma Dev) ; dotnet test → 135/135.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -561,8 +561,8 @@
 </file>
 
 <file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I30" headerRowCount="1">
-  <autoFilter ref="A4:I30"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I31" headerRowCount="1">
+  <autoFilter ref="A4:I31"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Code"/>
     <tableColumn id="2" name="Tâche"/>
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 15:00 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 15:11 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -2574,10 +2574,14 @@
       </c>
       <c r="H44" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
-        </is>
-      </c>
-      <c r="I44" s="5" t="inlineStr"/>
+          <t>EN_COURS</t>
+        </is>
+      </c>
+      <c r="I44" s="5" t="inlineStr">
+        <is>
+          <t>H-027</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="n">
@@ -14548,7 +14552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -15845,8 +15849,55 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>H-027</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>P1-T10</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>OUVERTE</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-16 15:11</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>Quels rôles déduire dans le socle, et comment traiter une délégation révoquée ?</t>
+        </is>
+      </c>
+      <c r="G31" s="5" t="inlineStr">
+        <is>
+          <t>Deux rôles déduits : RESPONSABLE_ENTITE (responsable d'une entité active) et DELEGATAIRE (délégation non supprimée couvrant aujourd'hui) ; révocation = suppression logique ; les rôles Directeur/Chef de division/Chef de service seront déduits du niveau de l'entité dans le module Organisation (P4). Hors requête et en Production avant P18 : utilisateur SYSTEME et 401 sur les contrôleurs</t>
+        </is>
+      </c>
+      <c r="H31" s="5" t="inlineStr">
+        <is>
+          <t>Enrichir DevAuthHandler si d'autres rôles sont requis ; prévoir un agent système en base si cree_par doit référencer un agent réel</t>
+        </is>
+      </c>
+      <c r="I31" s="5" t="inlineStr">
+        <is>
+          <t>en attente</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="C5:C30">
+  <conditionalFormatting sqref="C5:C31">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"NON_FAIT"</formula>
     </cfRule>
@@ -16767,7 +16818,7 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
@@ -16781,7 +16832,11 @@
         </is>
       </c>
       <c r="I17" s="5" t="inlineStr"/>
-      <c r="J17" s="5" t="inlineStr"/>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>H-027 (OUVERTE)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">

</xml_diff>

<commit_message>
P1-T11: Données de démonstration
database/04-donnees-demo.sql (1 direction, 3 divisions, 6 services, 25 agents fictifs A0001-A0025,
10 responsables, compétences, 2 délégations, 5 absences, 12 jours fériés 2026) ; option
pg-test.py demarrer --demo.
Test : 10 entités, 25 agents, 10 responsables, 6/6 services sous une division (ltree) ;
tester-schema 18/18 ; comparer-schema 0 écart ; dotnet test 135/135.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -561,8 +561,8 @@
 </file>
 
 <file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I31" headerRowCount="1">
-  <autoFilter ref="A4:I31"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I32" headerRowCount="1">
+  <autoFilter ref="A4:I32"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Code"/>
     <tableColumn id="2" name="Tâche"/>
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 15:14 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 15:18 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -2617,10 +2617,14 @@
       </c>
       <c r="H45" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
-        </is>
-      </c>
-      <c r="I45" s="5" t="inlineStr"/>
+          <t>EN_COURS</t>
+        </is>
+      </c>
+      <c r="I45" s="5" t="inlineStr">
+        <is>
+          <t>H-028</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="n">
@@ -14552,7 +14556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -15896,8 +15900,55 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>H-028</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>P1-T11</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>OUVERTE</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-16 15:18</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>Quels jours fériés 2026 retenir pour la démo, notamment les fêtes religieuses mobiles ?</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>Calendrier civil marocain pour les jours fixes ; fêtes mobiles 2026 à des dates indicatives (marquées « indicatif »), à confirmer par l'annonce officielle</t>
+        </is>
+      </c>
+      <c r="H32" s="5" t="inlineStr">
+        <is>
+          <t>Seules les données de démonstration seraient à corriger ; aucun calcul métier n'est encore branché dessus</t>
+        </is>
+      </c>
+      <c r="I32" s="5" t="inlineStr">
+        <is>
+          <t>en attente</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="C5:C31">
+  <conditionalFormatting sqref="C5:C32">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"NON_FAIT"</formula>
     </cfRule>
@@ -16864,7 +16915,7 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
@@ -16878,7 +16929,11 @@
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr"/>
-      <c r="J18" s="5" t="inlineStr"/>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>H-028 (OUVERTE)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
P1-T11: journal et statut de la tâche
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 15:18 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 15:19 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1121,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -2617,7 +2617,7 @@
       </c>
       <c r="H45" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="I45" s="5" t="inlineStr">
@@ -16346,7 +16346,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
     </row>
@@ -16915,7 +16915,7 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">

</xml_diff>

<commit_message>
P1: clôture de phase
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 15:19 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 15:35 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1121,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDEE</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -2191,7 +2191,7 @@
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="I35" s="5" t="inlineStr"/>
@@ -2230,7 +2230,7 @@
       </c>
       <c r="H36" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="I36" s="5" t="inlineStr">
@@ -2273,7 +2273,7 @@
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="I37" s="5" t="inlineStr">
@@ -2316,7 +2316,7 @@
       </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="I38" s="5" t="inlineStr">
@@ -2359,7 +2359,7 @@
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="I39" s="5" t="inlineStr">
@@ -2402,7 +2402,7 @@
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="I40" s="5" t="inlineStr">
@@ -2445,7 +2445,7 @@
       </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="I41" s="5" t="inlineStr">
@@ -2488,7 +2488,7 @@
       </c>
       <c r="H42" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="I42" s="5" t="inlineStr">
@@ -2531,7 +2531,7 @@
       </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="I43" s="5" t="inlineStr">
@@ -2574,7 +2574,7 @@
       </c>
       <c r="H44" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="I44" s="5" t="inlineStr">
@@ -2617,7 +2617,7 @@
       </c>
       <c r="H45" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="I45" s="5" t="inlineStr">
@@ -16346,7 +16346,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDEE</t>
         </is>
       </c>
     </row>
@@ -16458,7 +16458,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
@@ -16500,7 +16500,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
@@ -16546,7 +16546,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
@@ -16592,7 +16592,7 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
@@ -16638,7 +16638,7 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
@@ -16684,7 +16684,7 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
@@ -16730,7 +16730,7 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -16776,7 +16776,7 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
@@ -16822,7 +16822,7 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
@@ -16869,7 +16869,7 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
@@ -16915,7 +16915,7 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">

</xml_diff>

<commit_message>
P2-T01: Projet Gprojet-Front, hébergement par le backend et tests bUnit
src/Gprojet-Front (Blazor WASM, DTO en fichiers liés, arborescence des couches), servi par le backend
(ProjectReference sans types, UseBlazorFrameworkFiles, fallback hors api|health|openapi|scalar),
premier DTO SanteDto via GET /api/health, tests/Gprojet-Front.Tests (bUnit + règle d'architecture).
Test : build 0 avertissement ; 4 projets ; front 4/4 ; backend 143/143.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -561,8 +561,8 @@
 </file>
 
 <file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I32" headerRowCount="1">
-  <autoFilter ref="A4:I32"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I33" headerRowCount="1">
+  <autoFilter ref="A4:I33"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Code"/>
     <tableColumn id="2" name="Tâche"/>
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 15:35 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 15:42 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -1159,7 +1159,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>NON_DEMARREE</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -2660,10 +2660,14 @@
       </c>
       <c r="H46" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
-        </is>
-      </c>
-      <c r="I46" s="5" t="inlineStr"/>
+          <t>EN_COURS</t>
+        </is>
+      </c>
+      <c r="I46" s="5" t="inlineStr">
+        <is>
+          <t>H-029</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="n">
@@ -14556,7 +14560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:I33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -15947,8 +15951,55 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>H-029</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>P2-T01</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>OUVERTE</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-16 15:42</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>Quel premier DTO partagé, et où exposer la santé pour le front ?</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="inlineStr">
+        <is>
+          <t>SanteDto (record Statut) renvoyé par GET /api/health (minimal API anonyme), consommé par SanteApiClient ; /health et /health/ready restent pour l'exploitation</t>
+        </is>
+      </c>
+      <c r="H33" s="5" t="inlineStr">
+        <is>
+          <t>Renommage ou déplacement minime si un autre DTO de référence est préféré</t>
+        </is>
+      </c>
+      <c r="I33" s="5" t="inlineStr">
+        <is>
+          <t>en attente</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="C5:C32">
+  <conditionalFormatting sqref="C5:C33">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"NON_FAIT"</formula>
     </cfRule>
@@ -17072,7 +17123,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>NON_DEMARREE</t>
+          <t>EN_COURS</t>
         </is>
       </c>
     </row>
@@ -17184,7 +17235,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
@@ -17198,7 +17249,11 @@
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr"/>
-      <c r="J8" s="5" t="inlineStr"/>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>H-029 (OUVERTE)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">

</xml_diff>

<commit_message>
P2-T01: journal et statut de la tâche
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 15:42 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 15:43 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -2660,7 +2660,7 @@
       </c>
       <c r="H46" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="I46" s="5" t="inlineStr">
@@ -17235,7 +17235,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">

</xml_diff>

<commit_message>
P2-T02: Charte HCP : intégration de app.css et des ressources
app.css = charte HCP avec Geist en @font-face local, app.gp.css (5 variantes de texte accessibles
H-014, badges de statut, classes manquantes), Font Awesome Free 6.7.2 et Chart.js 4.5.1 auto-hébergés,
logo HCP, scripts/verifier-charte.py, docs/DESIGN.md.
Test : verifier-charte OK ; aucune URL externe ; Charte 3/3 (contrastes ≥ 4,5:1) ; front 7/7 ; backend 143/143.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -561,8 +561,8 @@
 </file>
 
 <file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I33" headerRowCount="1">
-  <autoFilter ref="A4:I33"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I34" headerRowCount="1">
+  <autoFilter ref="A4:I34"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Code"/>
     <tableColumn id="2" name="Tâche"/>
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 15:43 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 15:47 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -2703,12 +2703,12 @@
       </c>
       <c r="H47" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="I47" s="5" t="inlineStr">
         <is>
-          <t>H-014</t>
+          <t>H-014, H-030</t>
         </is>
       </c>
     </row>
@@ -14560,7 +14560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I33"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -15998,8 +15998,55 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>H-030</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>P2-T02</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>OUVERTE</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-16 15:47</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>Quelles classes de badge de statut prévoir, et comment mapper les statuts configurables de tâche/ticket ?</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>Classes kebab-case déduites des enums de statut du backend ; les workflows configurables (CategorieStatut) se mappent sur a-faire / en-cours / termine ; d'autres classes s'ajouteront au besoin</t>
+        </is>
+      </c>
+      <c r="H34" s="5" t="inlineStr">
+        <is>
+          <t>Ajout de classes dans app.gp.css si un statut n'est pas couvert</t>
+        </is>
+      </c>
+      <c r="I34" s="5" t="inlineStr">
+        <is>
+          <t>en attente</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="C5:C33">
+  <conditionalFormatting sqref="C5:C34">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"NON_FAIT"</formula>
     </cfRule>
@@ -17281,7 +17328,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
@@ -17297,7 +17344,8 @@
       <c r="I9" s="5" t="inlineStr"/>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>H-014 (REPONDUE)</t>
+          <t>H-014 (REPONDUE)
+H-030 (OUVERTE)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
P2-T02: journal et statut de la tâche
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 15:47 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 15:48 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -2703,7 +2703,7 @@
       </c>
       <c r="H47" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="I47" s="5" t="inlineStr">
@@ -17328,7 +17328,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">

</xml_diff>

<commit_message>
P2-T03: Layout principal et navigation par rôle
MainLayout conforme à la GED HCP (sidebar, topbar, content-area), menu filtré par politiques
(PortefeuilleDirection, Administration), repli et tiroir mobile (0.25s, prefers-reduced-motion),
Ctrl+K et lien d'évitement, rôles partagés dans Contracts/Commun/RolesApplication,
authentification front provisoire anonyme (shortcut).
Test : Category=Layout → 5/5 ; front 12/12 ; backend 143/143.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -561,8 +561,8 @@
 </file>
 
 <file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I34" headerRowCount="1">
-  <autoFilter ref="A4:I34"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I35" headerRowCount="1">
+  <autoFilter ref="A4:I35"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Code"/>
     <tableColumn id="2" name="Tâche"/>
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 15:48 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 15:52 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -2746,10 +2746,14 @@
       </c>
       <c r="H48" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
-        </is>
-      </c>
-      <c r="I48" s="5" t="inlineStr"/>
+          <t>EN_COURS</t>
+        </is>
+      </c>
+      <c r="I48" s="5" t="inlineStr">
+        <is>
+          <t>H-031</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="n">
@@ -14560,7 +14564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -16045,8 +16049,55 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>H-031</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>P2-T03</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>OUVERTE</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-16 15:52</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>Qui voit le menu Administration, et quand le rôle DIRECTEUR sera-t-il attribué ?</t>
+        </is>
+      </c>
+      <c r="G35" s="5" t="inlineStr">
+        <is>
+          <t>Administration = DIRECTEUR ou RESPONSABLE_ENTITE ; DIRECTEUR est déclaré (Contracts/Commun/RolesApplication) mais déduit côté serveur seulement en P4 ; libellés en dur en français tant que l'i18n (resx) n'existe pas</t>
+        </is>
+      </c>
+      <c r="H35" s="5" t="inlineStr">
+        <is>
+          <t>Politiques.cs à ajuster si besoin ; « Portefeuille direction » invisible pour tous jusqu'en P4 ; libellés à basculer en resx plus tard</t>
+        </is>
+      </c>
+      <c r="I35" s="5" t="inlineStr">
+        <is>
+          <t>en attente</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="C5:C34">
+  <conditionalFormatting sqref="C5:C35">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"NON_FAIT"</formula>
     </cfRule>
@@ -17375,7 +17426,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
@@ -17389,7 +17440,11 @@
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr"/>
-      <c r="J10" s="5" t="inlineStr"/>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>H-031 (OUVERTE)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">

</xml_diff>

<commit_message>
P2-T03: journal et statut de la tâche
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 15:52 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 15:53 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -2746,7 +2746,7 @@
       </c>
       <c r="H48" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="I48" s="5" t="inlineStr">
@@ -17426,7 +17426,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">

</xml_diff>

<commit_message>
P2-T04: Mouvement selon la charte (motion-design)
Seules les durées de la charte (0.1s, 0.15s, 0.25s, 0.6s) : .animate-in par route dans MainLayout,
règle dialogue fadeIn 0.25s, repli du menu 0.25s ; un bloc prefers-reduced-motion unique
(animation/transition: none) ; section Mouvement dans docs/DESIGN.md.
Test : Category=Mouvement → 3/3 ; grep des durées OK ; wwwroot/lib inchangé ; front 15/15 ; backend 143/143.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -2789,7 +2789,7 @@
       </c>
       <c r="H49" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="I49" s="5" t="inlineStr"/>
@@ -17472,7 +17472,7 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">

</xml_diff>

<commit_message>
P2-T04: journal et statut de la tâche
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 15:53 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 15:56 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -2789,7 +2789,7 @@
       </c>
       <c r="H49" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="I49" s="5" t="inlineStr"/>
@@ -17472,7 +17472,7 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">

</xml_diff>

<commit_message>
P2-T05: Couche Api : clients HTTP typés
ApiClientBase (System.Text.Json Web, Get/Post/Put/Delete avec annulation, ProblemDetails →
ApiException typée avec erreurs par champ, corps non JSON toléré), clients via IHttpClientFactory
en adresses relatives, SanteApiClient migré.
Test : Category=Api → 6/6 (200, 400 par champ, 404, 500 non JSON, annulation) ; front 21/21 ; backend 143/143.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -2828,7 +2828,7 @@
       </c>
       <c r="H50" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="I50" s="5" t="inlineStr"/>
@@ -17514,7 +17514,7 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">

</xml_diff>

<commit_message>
P2-T05: journal et statut de la tâche
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 15:56 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 15:58 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -2828,7 +2828,7 @@
       </c>
       <c r="H50" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="I50" s="5" t="inlineStr"/>
@@ -17514,7 +17514,7 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">

</xml_diff>

<commit_message>
P2-T06: journal et statut de la tâche
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 16:05 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 16:07 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -2867,7 +2867,7 @@
       </c>
       <c r="H51" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="I51" s="5" t="inlineStr">
@@ -17607,7 +17607,7 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">

</xml_diff>

<commit_message>
P2-T06: Authentification côté front (BFF, mode dev)
BFF /bff/login (dev, formulaire, redirection fixe), /bff/logout, /bff/user ; cookie gp.session
HttpOnly/Secure/SameSite=Strict, 401/403 sans redirection ; anti-CSRF global par en-tête X-CSRF: 1
sur les méthodes mutantes avec cookie ; IChargeurIdentite partagé avec DevAuthHandler ; Production :
aucun chemin d'authentification avant P18. Front : BffAuthenticationStateProvider, BffApiClient,
page /connexion, en-tête CSRF ajouté par ApiClientBase.
Test : backend 150/150 (dont 7 BFF) ; front 24/24 (dont 3 Auth).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -561,8 +561,8 @@
 </file>
 
 <file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I35" headerRowCount="1">
-  <autoFilter ref="A4:I35"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I36" headerRowCount="1">
+  <autoFilter ref="A4:I36"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Code"/>
     <tableColumn id="2" name="Tâche"/>
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 15:58 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 16:05 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -2867,10 +2867,14 @@
       </c>
       <c r="H51" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
-        </is>
-      </c>
-      <c r="I51" s="5" t="inlineStr"/>
+          <t>EN_COURS</t>
+        </is>
+      </c>
+      <c r="I51" s="5" t="inlineStr">
+        <is>
+          <t>H-032</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="n">
@@ -14564,7 +14568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:I36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -16096,8 +16100,55 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>H-032</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>P2-T06</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>OUVERTE</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-16 16:05</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>Les rôles sont-ils figés dans le cookie, et les pages doivent-elles rediriger les anonymes vers /connexion ?</t>
+        </is>
+      </c>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>Rôles lus au login et valables 8 h glissantes (shortcut jusqu'à Keycloak P18) ; pas de redirection automatique vers /connexion dans le socle, les gardes de pages viendront avec les pages métier ; anti-CSRF par en-tête X-CSRF: 1 obligatoire dès qu'un cookie de session est présent</t>
+        </is>
+      </c>
+      <c r="H36" s="5" t="inlineStr">
+        <is>
+          <t>Un changement de rôle ne s'applique qu'à la reconnexion ; ajouter des gardes de pages au besoin</t>
+        </is>
+      </c>
+      <c r="I36" s="5" t="inlineStr">
+        <is>
+          <t>en attente</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="C5:C35">
+  <conditionalFormatting sqref="C5:C36">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"NON_FAIT"</formula>
     </cfRule>
@@ -17556,7 +17607,7 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
@@ -17570,7 +17621,11 @@
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr"/>
-      <c r="J13" s="5" t="inlineStr"/>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>H-032 (OUVERTE)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">

</xml_diff>

<commit_message>
P2-T07: État partagé et services front de base
PerimetreState et UtilisateurCourantState (dérivé des claims), NotificationUiService + Snackbar
(role alert/status, disparition auto annulable), ChargementService + IndicateurChargement,
GestionnaireErreursUi (statut → message français, journal sans données sensibles).
Test : Category=Etat → 8/8 ; front 32/32 ; backend 150/150.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -561,8 +561,8 @@
 </file>
 
 <file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I36" headerRowCount="1">
-  <autoFilter ref="A4:I36"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I37" headerRowCount="1">
+  <autoFilter ref="A4:I37"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Code"/>
     <tableColumn id="2" name="Tâche"/>
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 16:07 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 16:10 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -2910,10 +2910,14 @@
       </c>
       <c r="H52" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
-        </is>
-      </c>
-      <c r="I52" s="5" t="inlineStr"/>
+          <t>EN_COURS</t>
+        </is>
+      </c>
+      <c r="I52" s="5" t="inlineStr">
+        <is>
+          <t>H-033</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="n">
@@ -14568,7 +14572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I36"/>
+  <dimension ref="A1:I37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -16147,8 +16151,55 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>H-033</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>P2-T07</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>OUVERTE</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-16 16:10</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>D'où viendront le niveau et le chemin du périmètre côté front, et quel délai de disparition des notifications ?</t>
+        </is>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>PerimetreState expose Definir(...) ; il sera alimenté par le module Organisation (P4), sans endpoint fantôme maintenant. Notifications : 6 s pour tous les types, réglable</t>
+        </is>
+      </c>
+      <c r="H37" s="5" t="inlineStr">
+        <is>
+          <t>Un endpoint ou un claim supplémentaire en P4 ; réglage simple du délai</t>
+        </is>
+      </c>
+      <c r="I37" s="5" t="inlineStr">
+        <is>
+          <t>en attente</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="C5:C36">
+  <conditionalFormatting sqref="C5:C37">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"NON_FAIT"</formula>
     </cfRule>
@@ -17653,7 +17704,7 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -17667,7 +17718,11 @@
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr"/>
-      <c r="J14" s="5" t="inlineStr"/>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>H-033 (OUVERTE)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">

</xml_diff>

<commit_message>
P2-T07: journal et statut de la tâche
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 16:10 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 16:11 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -2910,7 +2910,7 @@
       </c>
       <c r="H52" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="I52" s="5" t="inlineStr">
@@ -17704,7 +17704,7 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">

</xml_diff>

<commit_message>
P2-T08: Internationalisation fr / en / ar (RTL)
Resources/Textes (fr-MA par défaut, en, ar-MA, 43 clés), IStringLocalizer, sélecteur de langue,
POST /bff/langue (liste blanche, cookie gp.culture), culture appliquée avant le premier rendu,
dir/lang sur <html> et le layout, règles RTL dans app.gp.css (menu à droite), données ICU complètes,
textes du layout, des composants et des pages migrés.
Test : Category=I18n → 11/11 ; front 43/43 ; backend 157/157.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -561,8 +561,8 @@
 </file>
 
 <file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I37" headerRowCount="1">
-  <autoFilter ref="A4:I37"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I38" headerRowCount="1">
+  <autoFilter ref="A4:I38"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Code"/>
     <tableColumn id="2" name="Tâche"/>
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 16:11 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 16:22 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -2953,10 +2953,14 @@
       </c>
       <c r="H53" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
-        </is>
-      </c>
-      <c r="I53" s="5" t="inlineStr"/>
+          <t>EN_COURS</t>
+        </is>
+      </c>
+      <c r="I53" s="5" t="inlineStr">
+        <is>
+          <t>H-034</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="n">
@@ -14572,7 +14576,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I37"/>
+  <dimension ref="A1:I38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -16198,8 +16202,55 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>H-034</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>P2-T08</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>OUVERTE</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-16 16:22</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="inlineStr">
+        <is>
+          <t>Culture par défaut, police arabe et relecture des traductions ?</t>
+        </is>
+      </c>
+      <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t>fr-MA par défaut (repli), en et ar-MA ; arabe affiché avec la pile système (Geist sans glyphes arabes, aucune police téléchargée) ; traductions en/ar rédigées sans relecture native</t>
+        </is>
+      </c>
+      <c r="H38" s="5" t="inlineStr">
+        <is>
+          <t>Changer Langues.Defaut ; ajouter une police arabe auto-hébergée si le rendu système déplaît ; faire relire en et ar avant la mise en production</t>
+        </is>
+      </c>
+      <c r="I38" s="5" t="inlineStr">
+        <is>
+          <t>en attente</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="C5:C37">
+  <conditionalFormatting sqref="C5:C38">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"NON_FAIT"</formula>
     </cfRule>
@@ -17750,7 +17801,7 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
@@ -17764,7 +17815,11 @@
         </is>
       </c>
       <c r="I15" s="5" t="inlineStr"/>
-      <c r="J15" s="5" t="inlineStr"/>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>H-034 (OUVERTE)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">

</xml_diff>

<commit_message>
P2-T08: journal et statut de la tâche
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 16:22 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 16:23 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -2953,7 +2953,7 @@
       </c>
       <c r="H53" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="I53" s="5" t="inlineStr">
@@ -17801,7 +17801,7 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">

</xml_diff>

<commit_message>
P2-T09: journal et statut de la tâche
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 16:26 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 16:27 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -1159,7 +1159,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -2996,7 +2996,7 @@
       </c>
       <c r="H54" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="I54" s="5" t="inlineStr">
@@ -17425,7 +17425,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
     </row>
@@ -17898,7 +17898,7 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">

</xml_diff>

<commit_message>
P2: clôture de phase
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 16/10/2026 16:27 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 19/10/2026 09:42 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -1159,7 +1159,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDEE</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -2660,7 +2660,7 @@
       </c>
       <c r="H46" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="I46" s="5" t="inlineStr">
@@ -2703,7 +2703,7 @@
       </c>
       <c r="H47" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="I47" s="5" t="inlineStr">
@@ -2746,7 +2746,7 @@
       </c>
       <c r="H48" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="I48" s="5" t="inlineStr">
@@ -2789,7 +2789,7 @@
       </c>
       <c r="H49" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="I49" s="5" t="inlineStr"/>
@@ -2828,7 +2828,7 @@
       </c>
       <c r="H50" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="I50" s="5" t="inlineStr"/>
@@ -2867,7 +2867,7 @@
       </c>
       <c r="H51" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="I51" s="5" t="inlineStr">
@@ -2910,7 +2910,7 @@
       </c>
       <c r="H52" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="I52" s="5" t="inlineStr">
@@ -2953,7 +2953,7 @@
       </c>
       <c r="H53" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="I53" s="5" t="inlineStr">
@@ -2996,7 +2996,7 @@
       </c>
       <c r="H54" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="I54" s="5" t="inlineStr">
@@ -17425,7 +17425,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDEE</t>
         </is>
       </c>
     </row>
@@ -17537,7 +17537,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
@@ -17583,7 +17583,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
@@ -17630,7 +17630,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
@@ -17676,7 +17676,7 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
@@ -17718,7 +17718,7 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
@@ -17760,7 +17760,7 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
@@ -17806,7 +17806,7 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -17852,7 +17852,7 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
@@ -17898,7 +17898,7 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">

</xml_diff>

<commit_message>
backlog_excel : valeurs calculées au lieu de formules
Sur un poste sans Excel ni LibreOffice, les formules d'avancement
(COUNTIF) n'avaient pas de valeur en cache et s'affichaient vides ou à 0,
ce qui faisait paraître P1 non faite. Le classeur étant régénéré à chaque
transition, les valeurs sont désormais écrites directement.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 19/10/2026 09:42 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 19/10/2026 09:47 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -1091,21 +1091,17 @@
           <t>sonnet</t>
         </is>
       </c>
-      <c r="E5" s="4">
-        <f>COUNTA('P0'!B8:B200)</f>
-        <v/>
-      </c>
-      <c r="F5" s="4">
-        <f>COUNTIF('P0'!F8:F200,"A_VALIDER")+COUNTIF('P0'!F8:F200,"VALIDE")</f>
-        <v/>
-      </c>
-      <c r="G5" s="6">
-        <f>IF(E5=0,0,F5/E5)</f>
-        <v/>
-      </c>
-      <c r="H5" s="4">
-        <f>COUNTIF('P0'!F8:F200,"BLOQUE")</f>
-        <v/>
+      <c r="E5" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -1129,21 +1125,17 @@
           <t>opus</t>
         </is>
       </c>
-      <c r="E6" s="4">
-        <f>COUNTA('P1'!B8:B200)</f>
-        <v/>
-      </c>
-      <c r="F6" s="4">
-        <f>COUNTIF('P1'!F8:F200,"A_VALIDER")+COUNTIF('P1'!F8:F200,"VALIDE")</f>
-        <v/>
-      </c>
-      <c r="G6" s="6">
-        <f>IF(E6=0,0,F6/E6)</f>
-        <v/>
-      </c>
-      <c r="H6" s="4">
-        <f>COUNTIF('P1'!F8:F200,"BLOQUE")</f>
-        <v/>
+      <c r="E6" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -1167,21 +1159,17 @@
           <t>sonnet</t>
         </is>
       </c>
-      <c r="E7" s="4">
-        <f>COUNTA('P2'!B8:B200)</f>
-        <v/>
-      </c>
-      <c r="F7" s="4">
-        <f>COUNTIF('P2'!F8:F200,"A_VALIDER")+COUNTIF('P2'!F8:F200,"VALIDE")</f>
-        <v/>
-      </c>
-      <c r="G7" s="6">
-        <f>IF(E7=0,0,F7/E7)</f>
-        <v/>
-      </c>
-      <c r="H7" s="4">
-        <f>COUNTIF('P2'!F8:F200,"BLOQUE")</f>
-        <v/>
+      <c r="E7" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -1205,21 +1193,17 @@
           <t>sonnet</t>
         </is>
       </c>
-      <c r="E8" s="4">
-        <f>COUNTA('P3'!B8:B200)</f>
-        <v/>
-      </c>
-      <c r="F8" s="4">
-        <f>COUNTIF('P3'!F8:F200,"A_VALIDER")+COUNTIF('P3'!F8:F200,"VALIDE")</f>
-        <v/>
-      </c>
-      <c r="G8" s="6">
-        <f>IF(E8=0,0,F8/E8)</f>
-        <v/>
-      </c>
-      <c r="H8" s="4">
-        <f>COUNTIF('P3'!F8:F200,"BLOQUE")</f>
-        <v/>
+      <c r="E8" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -1243,21 +1227,17 @@
           <t>sonnet</t>
         </is>
       </c>
-      <c r="E9" s="4">
-        <f>COUNTA('P4'!B8:B200)</f>
-        <v/>
-      </c>
-      <c r="F9" s="4">
-        <f>COUNTIF('P4'!F8:F200,"A_VALIDER")+COUNTIF('P4'!F8:F200,"VALIDE")</f>
-        <v/>
-      </c>
-      <c r="G9" s="6">
-        <f>IF(E9=0,0,F9/E9)</f>
-        <v/>
-      </c>
-      <c r="H9" s="4">
-        <f>COUNTIF('P4'!F8:F200,"BLOQUE")</f>
-        <v/>
+      <c r="E9" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -1281,21 +1261,17 @@
           <t>opus</t>
         </is>
       </c>
-      <c r="E10" s="4">
-        <f>COUNTA('P5'!B8:B200)</f>
-        <v/>
-      </c>
-      <c r="F10" s="4">
-        <f>COUNTIF('P5'!F8:F200,"A_VALIDER")+COUNTIF('P5'!F8:F200,"VALIDE")</f>
-        <v/>
-      </c>
-      <c r="G10" s="6">
-        <f>IF(E10=0,0,F10/E10)</f>
-        <v/>
-      </c>
-      <c r="H10" s="4">
-        <f>COUNTIF('P5'!F8:F200,"BLOQUE")</f>
-        <v/>
+      <c r="E10" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -1319,21 +1295,17 @@
           <t>opus</t>
         </is>
       </c>
-      <c r="E11" s="4">
-        <f>COUNTA('P6'!B8:B200)</f>
-        <v/>
-      </c>
-      <c r="F11" s="4">
-        <f>COUNTIF('P6'!F8:F200,"A_VALIDER")+COUNTIF('P6'!F8:F200,"VALIDE")</f>
-        <v/>
-      </c>
-      <c r="G11" s="6">
-        <f>IF(E11=0,0,F11/E11)</f>
-        <v/>
-      </c>
-      <c r="H11" s="4">
-        <f>COUNTIF('P6'!F8:F200,"BLOQUE")</f>
-        <v/>
+      <c r="E11" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -1357,21 +1329,17 @@
           <t>sonnet</t>
         </is>
       </c>
-      <c r="E12" s="4">
-        <f>COUNTA('P7'!B8:B200)</f>
-        <v/>
-      </c>
-      <c r="F12" s="4">
-        <f>COUNTIF('P7'!F8:F200,"A_VALIDER")+COUNTIF('P7'!F8:F200,"VALIDE")</f>
-        <v/>
-      </c>
-      <c r="G12" s="6">
-        <f>IF(E12=0,0,F12/E12)</f>
-        <v/>
-      </c>
-      <c r="H12" s="4">
-        <f>COUNTIF('P7'!F8:F200,"BLOQUE")</f>
-        <v/>
+      <c r="E12" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -1395,21 +1363,17 @@
           <t>sonnet</t>
         </is>
       </c>
-      <c r="E13" s="4">
-        <f>COUNTA('P8'!B8:B200)</f>
-        <v/>
-      </c>
-      <c r="F13" s="4">
-        <f>COUNTIF('P8'!F8:F200,"A_VALIDER")+COUNTIF('P8'!F8:F200,"VALIDE")</f>
-        <v/>
-      </c>
-      <c r="G13" s="6">
-        <f>IF(E13=0,0,F13/E13)</f>
-        <v/>
-      </c>
-      <c r="H13" s="4">
-        <f>COUNTIF('P8'!F8:F200,"BLOQUE")</f>
-        <v/>
+      <c r="E13" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -1433,21 +1397,17 @@
           <t>sonnet</t>
         </is>
       </c>
-      <c r="E14" s="4">
-        <f>COUNTA('P9'!B8:B200)</f>
-        <v/>
-      </c>
-      <c r="F14" s="4">
-        <f>COUNTIF('P9'!F8:F200,"A_VALIDER")+COUNTIF('P9'!F8:F200,"VALIDE")</f>
-        <v/>
-      </c>
-      <c r="G14" s="6">
-        <f>IF(E14=0,0,F14/E14)</f>
-        <v/>
-      </c>
-      <c r="H14" s="4">
-        <f>COUNTIF('P9'!F8:F200,"BLOQUE")</f>
-        <v/>
+      <c r="E14" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -1471,21 +1431,17 @@
           <t>opus</t>
         </is>
       </c>
-      <c r="E15" s="4">
-        <f>COUNTA('P10'!B8:B200)</f>
-        <v/>
-      </c>
-      <c r="F15" s="4">
-        <f>COUNTIF('P10'!F8:F200,"A_VALIDER")+COUNTIF('P10'!F8:F200,"VALIDE")</f>
-        <v/>
-      </c>
-      <c r="G15" s="6">
-        <f>IF(E15=0,0,F15/E15)</f>
-        <v/>
-      </c>
-      <c r="H15" s="4">
-        <f>COUNTIF('P10'!F8:F200,"BLOQUE")</f>
-        <v/>
+      <c r="E15" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="F15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -1509,21 +1465,17 @@
           <t>opus</t>
         </is>
       </c>
-      <c r="E16" s="4">
-        <f>COUNTA('P11'!B8:B200)</f>
-        <v/>
-      </c>
-      <c r="F16" s="4">
-        <f>COUNTIF('P11'!F8:F200,"A_VALIDER")+COUNTIF('P11'!F8:F200,"VALIDE")</f>
-        <v/>
-      </c>
-      <c r="G16" s="6">
-        <f>IF(E16=0,0,F16/E16)</f>
-        <v/>
-      </c>
-      <c r="H16" s="4">
-        <f>COUNTIF('P11'!F8:F200,"BLOQUE")</f>
-        <v/>
+      <c r="E16" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -1547,21 +1499,17 @@
           <t>sonnet</t>
         </is>
       </c>
-      <c r="E17" s="4">
-        <f>COUNTA('P12'!B8:B200)</f>
-        <v/>
-      </c>
-      <c r="F17" s="4">
-        <f>COUNTIF('P12'!F8:F200,"A_VALIDER")+COUNTIF('P12'!F8:F200,"VALIDE")</f>
-        <v/>
-      </c>
-      <c r="G17" s="6">
-        <f>IF(E17=0,0,F17/E17)</f>
-        <v/>
-      </c>
-      <c r="H17" s="4">
-        <f>COUNTIF('P12'!F8:F200,"BLOQUE")</f>
-        <v/>
+      <c r="E17" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="F17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -1585,21 +1533,17 @@
           <t>sonnet</t>
         </is>
       </c>
-      <c r="E18" s="4">
-        <f>COUNTA('P13'!B8:B200)</f>
-        <v/>
-      </c>
-      <c r="F18" s="4">
-        <f>COUNTIF('P13'!F8:F200,"A_VALIDER")+COUNTIF('P13'!F8:F200,"VALIDE")</f>
-        <v/>
-      </c>
-      <c r="G18" s="6">
-        <f>IF(E18=0,0,F18/E18)</f>
-        <v/>
-      </c>
-      <c r="H18" s="4">
-        <f>COUNTIF('P13'!F8:F200,"BLOQUE")</f>
-        <v/>
+      <c r="E18" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -1623,21 +1567,17 @@
           <t>sonnet</t>
         </is>
       </c>
-      <c r="E19" s="4">
-        <f>COUNTA('P14'!B8:B200)</f>
-        <v/>
-      </c>
-      <c r="F19" s="4">
-        <f>COUNTIF('P14'!F8:F200,"A_VALIDER")+COUNTIF('P14'!F8:F200,"VALIDE")</f>
-        <v/>
-      </c>
-      <c r="G19" s="6">
-        <f>IF(E19=0,0,F19/E19)</f>
-        <v/>
-      </c>
-      <c r="H19" s="4">
-        <f>COUNTIF('P14'!F8:F200,"BLOQUE")</f>
-        <v/>
+      <c r="E19" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -1661,21 +1601,17 @@
           <t>sonnet</t>
         </is>
       </c>
-      <c r="E20" s="4">
-        <f>COUNTA('P15'!B8:B200)</f>
-        <v/>
-      </c>
-      <c r="F20" s="4">
-        <f>COUNTIF('P15'!F8:F200,"A_VALIDER")+COUNTIF('P15'!F8:F200,"VALIDE")</f>
-        <v/>
-      </c>
-      <c r="G20" s="6">
-        <f>IF(E20=0,0,F20/E20)</f>
-        <v/>
-      </c>
-      <c r="H20" s="4">
-        <f>COUNTIF('P15'!F8:F200,"BLOQUE")</f>
-        <v/>
+      <c r="E20" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -1699,21 +1635,17 @@
           <t>sonnet</t>
         </is>
       </c>
-      <c r="E21" s="4">
-        <f>COUNTA('P16'!B8:B200)</f>
-        <v/>
-      </c>
-      <c r="F21" s="4">
-        <f>COUNTIF('P16'!F8:F200,"A_VALIDER")+COUNTIF('P16'!F8:F200,"VALIDE")</f>
-        <v/>
-      </c>
-      <c r="G21" s="6">
-        <f>IF(E21=0,0,F21/E21)</f>
-        <v/>
-      </c>
-      <c r="H21" s="4">
-        <f>COUNTIF('P16'!F8:F200,"BLOQUE")</f>
-        <v/>
+      <c r="E21" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="F21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -1737,21 +1669,17 @@
           <t>sonnet</t>
         </is>
       </c>
-      <c r="E22" s="4">
-        <f>COUNTA('P17'!B8:B200)</f>
-        <v/>
-      </c>
-      <c r="F22" s="4">
-        <f>COUNTIF('P17'!F8:F200,"A_VALIDER")+COUNTIF('P17'!F8:F200,"VALIDE")</f>
-        <v/>
-      </c>
-      <c r="G22" s="6">
-        <f>IF(E22=0,0,F22/E22)</f>
-        <v/>
-      </c>
-      <c r="H22" s="4">
-        <f>COUNTIF('P17'!F8:F200,"BLOQUE")</f>
-        <v/>
+      <c r="E22" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -1775,21 +1703,17 @@
           <t>opus</t>
         </is>
       </c>
-      <c r="E23" s="4">
-        <f>COUNTA('P18'!B8:B200)</f>
-        <v/>
-      </c>
-      <c r="F23" s="4">
-        <f>COUNTIF('P18'!F8:F200,"A_VALIDER")+COUNTIF('P18'!F8:F200,"VALIDE")</f>
-        <v/>
-      </c>
-      <c r="G23" s="6">
-        <f>IF(E23=0,0,F23/E23)</f>
-        <v/>
-      </c>
-      <c r="H23" s="4">
-        <f>COUNTIF('P18'!F8:F200,"BLOQUE")</f>
-        <v/>
+      <c r="E23" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -1813,21 +1737,17 @@
           <t>sonnet</t>
         </is>
       </c>
-      <c r="E24" s="4">
-        <f>COUNTA('P19'!B8:B200)</f>
-        <v/>
-      </c>
-      <c r="F24" s="4">
-        <f>COUNTIF('P19'!F8:F200,"A_VALIDER")+COUNTIF('P19'!F8:F200,"VALIDE")</f>
-        <v/>
-      </c>
-      <c r="G24" s="6">
-        <f>IF(E24=0,0,F24/E24)</f>
-        <v/>
-      </c>
-      <c r="H24" s="4">
-        <f>COUNTIF('P19'!F8:F200,"BLOQUE")</f>
-        <v/>
+      <c r="E24" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="F24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -1836,21 +1756,17 @@
           <t>Total</t>
         </is>
       </c>
-      <c r="E25" s="8">
-        <f>SUM(E5:E24)</f>
-        <v/>
-      </c>
-      <c r="F25" s="8">
-        <f>SUM(F5:F24)</f>
-        <v/>
-      </c>
-      <c r="G25" s="9">
-        <f>IF(E25=0,0,F25/E25)</f>
-        <v/>
-      </c>
-      <c r="H25" s="8">
-        <f>SUM(H5:H24)</f>
-        <v/>
+      <c r="E25" s="8" t="n">
+        <v>148</v>
+      </c>
+      <c r="F25" s="8" t="n">
+        <v>26</v>
+      </c>
+      <c r="G25" s="9" t="n">
+        <v>0.1756756756756757</v>
+      </c>
+      <c r="H25" s="8" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -8124,9 +8040,8 @@
           <t>Avancement</t>
         </is>
       </c>
-      <c r="B5" s="12">
-        <f>IF(COUNTA(B8:B200)=0,0,(COUNTIF(F8:F200,"A_VALIDER")+COUNTIF(F8:F200,"VALIDE"))/COUNTA(B8:B200))</f>
-        <v/>
+      <c r="B5" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -8688,9 +8603,8 @@
           <t>Avancement</t>
         </is>
       </c>
-      <c r="B5" s="12">
-        <f>IF(COUNTA(B8:B200)=0,0,(COUNTIF(F8:F200,"A_VALIDER")+COUNTIF(F8:F200,"VALIDE"))/COUNTA(B8:B200))</f>
-        <v/>
+      <c r="B5" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -9125,9 +9039,8 @@
           <t>Avancement</t>
         </is>
       </c>
-      <c r="B5" s="12">
-        <f>IF(COUNTA(B8:B200)=0,0,(COUNTIF(F8:F200,"A_VALIDER")+COUNTIF(F8:F200,"VALIDE"))/COUNTA(B8:B200))</f>
-        <v/>
+      <c r="B5" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -9734,9 +9647,8 @@
           <t>Avancement</t>
         </is>
       </c>
-      <c r="B5" s="12">
-        <f>IF(COUNTA(B8:B200)=0,0,(COUNTIF(F8:F200,"A_VALIDER")+COUNTIF(F8:F200,"VALIDE"))/COUNTA(B8:B200))</f>
-        <v/>
+      <c r="B5" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -10251,9 +10163,8 @@
           <t>Avancement</t>
         </is>
       </c>
-      <c r="B5" s="12">
-        <f>IF(COUNTA(B8:B200)=0,0,(COUNTIF(F8:F200,"A_VALIDER")+COUNTIF(F8:F200,"VALIDE"))/COUNTA(B8:B200))</f>
-        <v/>
+      <c r="B5" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -10730,9 +10641,8 @@
           <t>Avancement</t>
         </is>
       </c>
-      <c r="B5" s="12">
-        <f>IF(COUNTA(B8:B200)=0,0,(COUNTIF(F8:F200,"A_VALIDER")+COUNTIF(F8:F200,"VALIDE"))/COUNTA(B8:B200))</f>
-        <v/>
+      <c r="B5" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -11163,9 +11073,8 @@
           <t>Avancement</t>
         </is>
       </c>
-      <c r="B5" s="12">
-        <f>IF(COUNTA(B8:B200)=0,0,(COUNTIF(F8:F200,"A_VALIDER")+COUNTIF(F8:F200,"VALIDE"))/COUNTA(B8:B200))</f>
-        <v/>
+      <c r="B5" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -11638,9 +11547,8 @@
           <t>Avancement</t>
         </is>
       </c>
-      <c r="B5" s="12">
-        <f>IF(COUNTA(B8:B200)=0,0,(COUNTIF(F8:F200,"A_VALIDER")+COUNTIF(F8:F200,"VALIDE"))/COUNTA(B8:B200))</f>
-        <v/>
+      <c r="B5" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -12117,9 +12025,8 @@
           <t>Avancement</t>
         </is>
       </c>
-      <c r="B5" s="12">
-        <f>IF(COUNTA(B8:B200)=0,0,(COUNTIF(F8:F200,"A_VALIDER")+COUNTIF(F8:F200,"VALIDE"))/COUNTA(B8:B200))</f>
-        <v/>
+      <c r="B5" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -12592,9 +12499,8 @@
           <t>Avancement</t>
         </is>
       </c>
-      <c r="B5" s="12">
-        <f>IF(COUNTA(B8:B200)=0,0,(COUNTIF(F8:F200,"A_VALIDER")+COUNTIF(F8:F200,"VALIDE"))/COUNTA(B8:B200))</f>
-        <v/>
+      <c r="B5" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -13151,9 +13057,8 @@
           <t>Avancement</t>
         </is>
       </c>
-      <c r="B5" s="12">
-        <f>IF(COUNTA(B8:B200)=0,0,(COUNTIF(F8:F200,"A_VALIDER")+COUNTIF(F8:F200,"VALIDE"))/COUNTA(B8:B200))</f>
-        <v/>
+      <c r="B5" s="12" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -13643,9 +13548,8 @@
           <t>Avancement</t>
         </is>
       </c>
-      <c r="B5" s="12">
-        <f>IF(COUNTA(B8:B200)=0,0,(COUNTIF(F8:F200,"A_VALIDER")+COUNTIF(F8:F200,"VALIDE"))/COUNTA(B8:B200))</f>
-        <v/>
+      <c r="B5" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -14164,9 +14068,8 @@
           <t>Avancement</t>
         </is>
       </c>
-      <c r="B5" s="12">
-        <f>IF(COUNTA(B8:B200)=0,0,(COUNTIF(F8:F200,"A_VALIDER")+COUNTIF(F8:F200,"VALIDE"))/COUNTA(B8:B200))</f>
-        <v/>
+      <c r="B5" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -16721,9 +16624,8 @@
           <t>Avancement</t>
         </is>
       </c>
-      <c r="B5" s="12">
-        <f>IF(COUNTA(B8:B200)=0,0,(COUNTIF(F8:F200,"A_VALIDER")+COUNTIF(F8:F200,"VALIDE"))/COUNTA(B8:B200))</f>
-        <v/>
+      <c r="B5" s="12" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -17447,9 +17349,8 @@
           <t>Avancement</t>
         </is>
       </c>
-      <c r="B5" s="12">
-        <f>IF(COUNTA(B8:B200)=0,0,(COUNTIF(F8:F200,"A_VALIDER")+COUNTIF(F8:F200,"VALIDE"))/COUNTA(B8:B200))</f>
-        <v/>
+      <c r="B5" s="12" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -18077,9 +17978,8 @@
           <t>Avancement</t>
         </is>
       </c>
-      <c r="B5" s="12">
-        <f>IF(COUNTA(B8:B200)=0,0,(COUNTIF(F8:F200,"A_VALIDER")+COUNTIF(F8:F200,"VALIDE"))/COUNTA(B8:B200))</f>
-        <v/>
+      <c r="B5" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -18518,9 +18418,8 @@
           <t>Avancement</t>
         </is>
       </c>
-      <c r="B5" s="12">
-        <f>IF(COUNTA(B8:B200)=0,0,(COUNTIF(F8:F200,"A_VALIDER")+COUNTIF(F8:F200,"VALIDE"))/COUNTA(B8:B200))</f>
-        <v/>
+      <c r="B5" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -19077,9 +18976,8 @@
           <t>Avancement</t>
         </is>
       </c>
-      <c r="B5" s="12">
-        <f>IF(COUNTA(B8:B200)=0,0,(COUNTIF(F8:F200,"A_VALIDER")+COUNTIF(F8:F200,"VALIDE"))/COUNTA(B8:B200))</f>
-        <v/>
+      <c r="B5" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -19720,9 +19618,8 @@
           <t>Avancement</t>
         </is>
       </c>
-      <c r="B5" s="12">
-        <f>IF(COUNTA(B8:B200)=0,0,(COUNTIF(F8:F200,"A_VALIDER")+COUNTIF(F8:F200,"VALIDE"))/COUNTA(B8:B200))</f>
-        <v/>
+      <c r="B5" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -20451,9 +20348,8 @@
           <t>Avancement</t>
         </is>
       </c>
-      <c r="B5" s="12">
-        <f>IF(COUNTA(B8:B200)=0,0,(COUNTIF(F8:F200,"A_VALIDER")+COUNTIF(F8:F200,"VALIDE"))/COUNTA(B8:B200))</f>
-        <v/>
+      <c r="B5" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
P3-T01: Dockerfile de l'application
Dockerfile multi-étapes (sdk:10.0 -> aspnet:10.0-alpine + ICU), utilisateur non-root (1654), HEALTHCHECK /health, .dockerignore.
Test : docker build OK ; id -u = 1654 ; wwwroot/_framework présent ; image 259MB ; healthcheck healthy.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 19/10/2026 09:47 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 21/10/2026 10:51 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -1185,7 +1185,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>NON_DEMARREE</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -2955,7 +2955,7 @@
       </c>
       <c r="H55" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="I55" s="5" t="inlineStr">
@@ -17956,7 +17956,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>NON_DEMARREE</t>
+          <t>EN_COURS</t>
         </is>
       </c>
     </row>
@@ -18067,7 +18067,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">

</xml_diff>

<commit_message>
P3-T01: journal et statut de la tâche
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 21/10/2026 10:51 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 21/10/2026 10:58 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -1197,10 +1197,10 @@
         <v>5</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="H8" s="4" t="n">
         <v>0</v>
@@ -1760,10 +1760,10 @@
         <v>148</v>
       </c>
       <c r="F25" s="8" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>0.1756756756756757</v>
+        <v>0.1824324324324324</v>
       </c>
       <c r="H25" s="8" t="n">
         <v>0</v>
@@ -2955,7 +2955,7 @@
       </c>
       <c r="H55" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="I55" s="5" t="inlineStr">
@@ -17979,7 +17979,7 @@
         </is>
       </c>
       <c r="B5" s="12" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="6">
@@ -18067,7 +18067,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">

</xml_diff>

<commit_message>
P3-T02: journal et statut de la tâche
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 21/10/2026 11:03 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 21/10/2026 11:04 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -1197,10 +1197,10 @@
         <v>5</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="H8" s="4" t="n">
         <v>0</v>
@@ -1760,10 +1760,10 @@
         <v>148</v>
       </c>
       <c r="F25" s="8" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>0.1824324324324324</v>
+        <v>0.1891891891891892</v>
       </c>
       <c r="H25" s="8" t="n">
         <v>0</v>
@@ -2998,7 +2998,7 @@
       </c>
       <c r="H56" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="I56" s="5" t="inlineStr">
@@ -18030,7 +18030,7 @@
         </is>
       </c>
       <c r="B5" s="12" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="6">
@@ -18164,7 +18164,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">

</xml_diff>

<commit_message>
P3-T02: docker compose de développement
deploy/docker-compose.yml : postgres:18 (volume, port 55433), migrations (bundle EF, stage Dockerfile 'migrations'), app (final), profil keycloak, réseau gprojet ; deploy/.env.example sans secret.
Test : up -d --wait OK (APP_HOST_PORT=18080, 8080 occupé — H-036) ; /api/health 200 ; / HTML ; 61 tables via le bundle ; down -v propre.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -561,8 +561,8 @@
 </file>
 
 <file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I39" headerRowCount="1">
-  <autoFilter ref="A4:I39"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I40" headerRowCount="1">
+  <autoFilter ref="A4:I40"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Code"/>
     <tableColumn id="2" name="Tâche"/>
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 21/10/2026 10:58 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 21/10/2026 11:03 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -2998,10 +2998,14 @@
       </c>
       <c r="H56" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
-        </is>
-      </c>
-      <c r="I56" s="5" t="inlineStr"/>
+          <t>EN_COURS</t>
+        </is>
+      </c>
+      <c r="I56" s="5" t="inlineStr">
+        <is>
+          <t>H-036</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="n">
@@ -14483,7 +14487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:I40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -16203,8 +16207,55 @@
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>H-036</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>P3-T02</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>OUVERTE</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-21 11:03</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>Le port 8080 du poste est occupé par un conteneur youtrack étranger au projet : faut-il changer le port par défaut de l'app dans le compose ?</t>
+        </is>
+      </c>
+      <c r="G40" s="5" t="inlineStr">
+        <is>
+          <t>Port par défaut 8080 conservé, surchargeable par APP_HOST_PORT dans deploy/.env ; tests faits sur 18080 sans arrêter youtrack.</t>
+        </is>
+      </c>
+      <c r="H40" s="5" t="inlineStr">
+        <is>
+          <t>Avec youtrack actif, http://localhost:8080 répond YouTrack et non GestionProjet tant que APP_HOST_PORT n'est pas défini.</t>
+        </is>
+      </c>
+      <c r="I40" s="5" t="inlineStr">
+        <is>
+          <t>en attente</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="C5:C39">
+  <conditionalFormatting sqref="C5:C40">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"NON_FAIT"</formula>
     </cfRule>
@@ -18113,7 +18164,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
@@ -18127,7 +18178,11 @@
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr"/>
-      <c r="J9" s="5" t="inlineStr"/>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>H-036 (OUVERTE)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">

</xml_diff>

<commit_message>
P3-T03: Tests en CI avec PostgreSQL de service
PgTestFixture : GP_TEST_CONNECTION (serveur fourni par la CI) dérive les chaînes admin/jetable, pg-test.py non lancé, seule gp_it_* créée/migrée/supprimée, Database=gprojet refusée ; CONTRIBUTING.md.
Test : dotnet test local 157/157 + 50/50 ; GP_TEST_CONNECTION sur pg-test 157/157 ; postgres:18 avec mot de passe 157/157.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -3041,7 +3041,7 @@
       </c>
       <c r="H57" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="I57" s="5" t="inlineStr"/>
@@ -18210,7 +18210,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">

</xml_diff>

<commit_message>
P3-T03: journal et statut de la tâche
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 21/10/2026 11:04 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 21/10/2026 11:08 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -1197,10 +1197,10 @@
         <v>5</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="H8" s="4" t="n">
         <v>0</v>
@@ -1760,10 +1760,10 @@
         <v>148</v>
       </c>
       <c r="F25" s="8" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>0.1891891891891892</v>
+        <v>0.1959459459459459</v>
       </c>
       <c r="H25" s="8" t="n">
         <v>0</v>
@@ -3041,7 +3041,7 @@
       </c>
       <c r="H57" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="I57" s="5" t="inlineStr"/>
@@ -18030,7 +18030,7 @@
         </is>
       </c>
       <c r="B5" s="12" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="6">
@@ -18210,7 +18210,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">

</xml_diff>

<commit_message>
P3-T04: Workflow GitHub Actions
.github/workflows/ci.yml : build, test (postgres:18, GP_TEST_CONNECTION, TRX + couverture), qualite (dotnet format), securite (CodeQL, dependency-review, Trivy), paquet (ghcr.io, main/tags), deploiement (dispatch, environnement production) ; actions épinglées par SHA ; scripts/verifier-ci.py (+ --auto-test) ; coverlet.collector ; .editorconfig (champs privés static en PascalCase) et reformatage mécanique dotnet format ; case CI dans le modèle de PR.
Test : verifier-ci OK, auto-test 4 pièges rejetés ; build 0 avertissement ; format propre ; tests 157/157 + 50/50 ; comparer-schema 0 écart.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -561,8 +561,8 @@
 </file>
 
 <file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I40" headerRowCount="1">
-  <autoFilter ref="A4:I40"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I41" headerRowCount="1">
+  <autoFilter ref="A4:I41"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Code"/>
     <tableColumn id="2" name="Tâche"/>
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 21/10/2026 11:08 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 21/10/2026 11:16 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -3080,12 +3080,12 @@
       </c>
       <c r="H58" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="I58" s="5" t="inlineStr">
         <is>
-          <t>H-002</t>
+          <t>H-002, H-037</t>
         </is>
       </c>
     </row>
@@ -14487,7 +14487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I40"/>
+  <dimension ref="A1:I41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -16254,8 +16254,55 @@
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>H-037</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>P3-T04</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>OUVERTE</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-21 11:16</t>
+        </is>
+      </c>
+      <c r="F41" s="5" t="inlineStr">
+        <is>
+          <t>Les versions d'actions épinglées et le comportement réel du workflow (Trivy bloquant sur CRITICAL/HIGH, environnement production) ne peuvent être constatés qu'après le push : faut-il assouplir Trivy ?</t>
+        </is>
+      </c>
+      <c r="G41" s="5" t="inlineStr">
+        <is>
+          <t>Trivy bloquant (exit-code 1, CRITICAL/HIGH, unfixed ignorés) ; environnement 'production' à créer dans les réglages GitHub avec relecteurs ; déploiement manuel lancé depuis main ; actions épinglées par SHA (checkout v4.2.2, etc.).</t>
+        </is>
+      </c>
+      <c r="H41" s="5" t="inlineStr">
+        <is>
+          <t>Premier run possiblement rouge (vulnérabilité de l'image de base, version d'action) : à corriger après le premier push.</t>
+        </is>
+      </c>
+      <c r="I41" s="5" t="inlineStr">
+        <is>
+          <t>en attente</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="C5:C40">
+  <conditionalFormatting sqref="C5:C41">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"NON_FAIT"</formula>
     </cfRule>
@@ -18252,7 +18299,7 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
@@ -18268,7 +18315,8 @@
       <c r="I11" s="5" t="inlineStr"/>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>H-002 (REPONDUE)</t>
+          <t>H-002 (REPONDUE)
+H-037 (OUVERTE)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
P3-T04: journal et statut de la tâche
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 21/10/2026 11:16 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 21/10/2026 11:17 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -1197,10 +1197,10 @@
         <v>5</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="H8" s="4" t="n">
         <v>0</v>
@@ -1760,10 +1760,10 @@
         <v>148</v>
       </c>
       <c r="F25" s="8" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>0.1959459459459459</v>
+        <v>0.2027027027027027</v>
       </c>
       <c r="H25" s="8" t="n">
         <v>0</v>
@@ -3080,7 +3080,7 @@
       </c>
       <c r="H58" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="I58" s="5" t="inlineStr">
@@ -18077,7 +18077,7 @@
         </is>
       </c>
       <c r="B5" s="12" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="6">
@@ -18299,7 +18299,7 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">

</xml_diff>

<commit_message>
P3-T05: Documentation de déploiement local
docs/DEPLOIEMENT.md : Prérequis, Variables, Démarrage, Migrations, Pipeline (6 jobs, ghcr.io, aucun secret requis, environnement production), Dépannage.
Test : 5 sections présentes ; chemins et commandes cités existent ; compose config -q OK ; up -d --wait + /api/health 200 + down -v rejoués.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -3123,7 +3123,7 @@
       </c>
       <c r="H59" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="I59" s="5" t="inlineStr"/>
@@ -18346,7 +18346,7 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>NON_FAIT</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">

</xml_diff>

<commit_message>
P3-T05: journal et statut de la tâche
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 21/10/2026 11:17 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 21/10/2026 11:20 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -1185,7 +1185,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -1197,10 +1197,10 @@
         <v>5</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="H8" s="4" t="n">
         <v>0</v>
@@ -1760,10 +1760,10 @@
         <v>148</v>
       </c>
       <c r="F25" s="8" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>0.2027027027027027</v>
+        <v>0.2094594594594595</v>
       </c>
       <c r="H25" s="8" t="n">
         <v>0</v>
@@ -3123,7 +3123,7 @@
       </c>
       <c r="H59" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="I59" s="5" t="inlineStr"/>
@@ -18054,7 +18054,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
     </row>
@@ -18077,7 +18077,7 @@
         </is>
       </c>
       <c r="B5" s="12" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -18346,7 +18346,7 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>EN_COURS</t>
+          <t>A_VALIDER</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">

</xml_diff>

<commit_message>
P3: clôture de phase
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 21/10/2026 11:20 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 21/10/2026 14:52 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -1185,7 +1185,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDEE</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -2955,7 +2955,7 @@
       </c>
       <c r="H55" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="I55" s="5" t="inlineStr">
@@ -2998,7 +2998,7 @@
       </c>
       <c r="H56" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="I56" s="5" t="inlineStr">
@@ -3041,7 +3041,7 @@
       </c>
       <c r="H57" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="I57" s="5" t="inlineStr"/>
@@ -3080,7 +3080,7 @@
       </c>
       <c r="H58" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="I58" s="5" t="inlineStr">
@@ -3123,7 +3123,7 @@
       </c>
       <c r="H59" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="I59" s="5" t="inlineStr"/>
@@ -18054,7 +18054,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDEE</t>
         </is>
       </c>
     </row>
@@ -18165,7 +18165,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
@@ -18211,7 +18211,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
@@ -18257,7 +18257,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
@@ -18299,7 +18299,7 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
@@ -18346,7 +18346,7 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>A_VALIDER</t>
+          <t>VALIDE</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Revert "Phase/p3 conteneurisation ci"
</commit_message>
<xml_diff>
--- a/backlog/BACKLOG.xlsx
+++ b/backlog/BACKLOG.xlsx
@@ -561,8 +561,8 @@
 </file>
 
 <file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I41" headerRowCount="1">
-  <autoFilter ref="A4:I41"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="Hypotheses" displayName="Hypotheses" ref="A4:I18" headerRowCount="1">
+  <autoFilter ref="A4:I18"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Code"/>
     <tableColumn id="2" name="Tâche"/>
@@ -1024,7 +1024,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Généré le 21/10/2026 14:52 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
+          <t>Généré le 16/10/2026 11:48 depuis backlog/BACKLOG.md. Ne pas modifier : les statuts changent via /lancer-phase, /valider-phase, /refuser-tache et scripts/backlog.py.</t>
         </is>
       </c>
     </row>
@@ -1083,7 +1083,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>VALIDEE</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -1091,17 +1091,21 @@
           <t>sonnet</t>
         </is>
       </c>
-      <c r="E5" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="F5" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="G5" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="H5" s="4" t="n">
-        <v>0</v>
+      <c r="E5" s="4">
+        <f>COUNTA('P0'!B8:B200)</f>
+        <v/>
+      </c>
+      <c r="F5" s="4">
+        <f>COUNTIF('P0'!F8:F200,"A_VALIDER")+COUNTIF('P0'!F8:F200,"VALIDE")</f>
+        <v/>
+      </c>
+      <c r="G5" s="6">
+        <f>IF(E5=0,0,F5/E5)</f>
+        <v/>
+      </c>
+      <c r="H5" s="4">
+        <f>COUNTIF('P0'!F8:F200,"BLOQUE")</f>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -1117,7 +1121,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>VALIDEE</t>
+          <t>NON_DEMARREE</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -1125,17 +1129,21 @@
           <t>opus</t>
         </is>
       </c>
-      <c r="E6" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="F6" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="G6" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="H6" s="4" t="n">
-        <v>0</v>
+      <c r="E6" s="4">
+        <f>COUNTA('P1'!B8:B200)</f>
+        <v/>
+      </c>
+      <c r="F6" s="4">
+        <f>COUNTIF('P1'!F8:F200,"A_VALIDER")+COUNTIF('P1'!F8:F200,"VALIDE")</f>
+        <v/>
+      </c>
+      <c r="G6" s="6">
+        <f>IF(E6=0,0,F6/E6)</f>
+        <v/>
+      </c>
+      <c r="H6" s="4">
+        <f>COUNTIF('P1'!F8:F200,"BLOQUE")</f>
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -1151,7 +1159,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>VALIDEE</t>
+          <t>NON_DEMARREE</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -1159,17 +1167,21 @@
           <t>sonnet</t>
         </is>
       </c>
-      <c r="E7" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="F7" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="G7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="H7" s="4" t="n">
-        <v>0</v>
+      <c r="E7" s="4">
+        <f>COUNTA('P2'!B8:B200)</f>
+        <v/>
+      </c>
+      <c r="F7" s="4">
+        <f>COUNTIF('P2'!F8:F200,"A_VALIDER")+COUNTIF('P2'!F8:F200,"VALIDE")</f>
+        <v/>
+      </c>
+      <c r="G7" s="6">
+        <f>IF(E7=0,0,F7/E7)</f>
+        <v/>
+      </c>
+      <c r="H7" s="4">
+        <f>COUNTIF('P2'!F8:F200,"BLOQUE")</f>
+        <v/>
       </c>
     </row>
     <row r="8">
@@ -1180,12 +1192,12 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Conteneurisation et intégration continue GitHub Actions</t>
+          <t>Conteneurisation et intégration continue GitLab</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>VALIDEE</t>
+          <t>NON_DEMARREE</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -1193,17 +1205,21 @@
           <t>sonnet</t>
         </is>
       </c>
-      <c r="E8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="F8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="G8" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="H8" s="4" t="n">
-        <v>0</v>
+      <c r="E8" s="4">
+        <f>COUNTA('P3'!B8:B200)</f>
+        <v/>
+      </c>
+      <c r="F8" s="4">
+        <f>COUNTIF('P3'!F8:F200,"A_VALIDER")+COUNTIF('P3'!F8:F200,"VALIDE")</f>
+        <v/>
+      </c>
+      <c r="G8" s="6">
+        <f>IF(E8=0,0,F8/E8)</f>
+        <v/>
+      </c>
+      <c r="H8" s="4">
+        <f>COUNTIF('P3'!F8:F200,"BLOQUE")</f>
+        <v/>
       </c>
     </row>
     <row r="9">
@@ -1227,17 +1243,21 @@
           <t>sonnet</t>
         </is>
       </c>
-      <c r="E9" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="F9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" s="4" t="n">
-        <v>0</v>
+      <c r="E9" s="4">
+        <f>COUNTA('P4'!B8:B200)</f>
+        <v/>
+      </c>
+      <c r="F9" s="4">
+        <f>COUNTIF('P4'!F8:F200,"A_VALIDER")+COUNTIF('P4'!F8:F200,"VALIDE")</f>
+        <v/>
+      </c>
+      <c r="G9" s="6">
+        <f>IF(E9=0,0,F9/E9)</f>
+        <v/>
+      </c>
+      <c r="H9" s="4">
+        <f>COUNTIF('P4'!F8:F200,"BLOQUE")</f>
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -1261,17 +1281,21 @@
           <t>opus</t>
         </is>
       </c>
-      <c r="E10" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="F10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="4" t="n">
-        <v>0</v>
+      <c r="E10" s="4">
+        <f>COUNTA('P5'!B8:B200)</f>
+        <v/>
+      </c>
+      <c r="F10" s="4">
+        <f>COUNTIF('P5'!F8:F200,"A_VALIDER")+COUNTIF('P5'!F8:F200,"VALIDE")</f>
+        <v/>
+      </c>
+      <c r="G10" s="6">
+        <f>IF(E10=0,0,F10/E10)</f>
+        <v/>
+      </c>
+      <c r="H10" s="4">
+        <f>COUNTIF('P5'!F8:F200,"BLOQUE")</f>
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -1295,17 +1319,21 @@
           <t>opus</t>
         </is>
       </c>
-      <c r="E11" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="F11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" s="4" t="n">
-        <v>0</v>
+      <c r="E11" s="4">
+        <f>COUNTA('P6'!B8:B200)</f>
+        <v/>
+      </c>
+      <c r="F11" s="4">
+        <f>COUNTIF('P6'!F8:F200,"A_VALIDER")+COUNTIF('P6'!F8:F200,"VALIDE")</f>
+        <v/>
+      </c>
+      <c r="G11" s="6">
+        <f>IF(E11=0,0,F11/E11)</f>
+        <v/>
+      </c>
+      <c r="H11" s="4">
+        <f>COUNTIF('P6'!F8:F200,"BLOQUE")</f>
+        <v/>
       </c>
     </row>
     <row r="12">
@@ -1329,17 +1357,21 @@
           <t>sonnet</t>
         </is>
       </c>
-      <c r="E12" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="F12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" s="4" t="n">
-        <v>0</v>
+      <c r="E12" s="4">
+        <f>COUNTA('P7'!B8:B200)</f>
+        <v/>
+      </c>
+      <c r="F12" s="4">
+        <f>COUNTIF('P7'!F8:F200,"A_VALIDER")+COUNTIF('P7'!F8:F200,"VALIDE")</f>
+        <v/>
+      </c>
+      <c r="G12" s="6">
+        <f>IF(E12=0,0,F12/E12)</f>
+        <v/>
+      </c>
+      <c r="H12" s="4">
+        <f>COUNTIF('P7'!F8:F200,"BLOQUE")</f>
+        <v/>
       </c>
     </row>
     <row r="13">
@@ -1363,17 +1395,21 @@
           <t>sonnet</t>
         </is>
       </c>
-      <c r="E13" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="F13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" s="4" t="n">
-        <v>0</v>
+      <c r="E13" s="4">
+        <f>COUNTA('P8'!B8:B200)</f>
+        <v/>
+      </c>
+      <c r="F13" s="4">
+        <f>COUNTIF('P8'!F8:F200,"A_VALIDER")+COUNTIF('P8'!F8:F200,"VALIDE")</f>
+        <v/>
+      </c>
+      <c r="G13" s="6">
+        <f>IF(E13=0,0,F13/E13)</f>
+        <v/>
+      </c>
+      <c r="H13" s="4">
+        <f>COUNTIF('P8'!F8:F200,"BLOQUE")</f>
+        <v/>
       </c>
     </row>
     <row r="14">
@@ -1397,17 +1433,21 @@
           <t>sonnet</t>
         </is>
       </c>
-      <c r="E14" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="F14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" s="4" t="n">
-        <v>0</v>
+      <c r="E14" s="4">
+        <f>COUNTA('P9'!B8:B200)</f>
+        <v/>
+      </c>
+      <c r="F14" s="4">
+        <f>COUNTIF('P9'!F8:F200,"A_VALIDER")+COUNTIF('P9'!F8:F200,"VALIDE")</f>
+        <v/>
+      </c>
+      <c r="G14" s="6">
+        <f>IF(E14=0,0,F14/E14)</f>
+        <v/>
+      </c>
+      <c r="H14" s="4">
+        <f>COUNTIF('P9'!F8:F200,"BLOQUE")</f>
+        <v/>
       </c>
     </row>
     <row r="15">
@@ -1431,17 +1471,21 @@
           <t>opus</t>
         </is>
       </c>
-      <c r="E15" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="F15" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" s="4" t="n">
-        <v>0</v>
+      <c r="E15" s="4">
+        <f>COUNTA('P10'!B8:B200)</f>
+        <v/>
+      </c>
+      <c r="F15" s="4">
+        <f>COUNTIF('P10'!F8:F200,"A_VALIDER")+COUNTIF('P10'!F8:F200,"VALIDE")</f>
+        <v/>
+      </c>
+      <c r="G15" s="6">
+        <f>IF(E15=0,0,F15/E15)</f>
+        <v/>
+      </c>
+      <c r="H15" s="4">
+        <f>COUNTIF('P10'!F8:F200,"BLOQUE")</f>
+        <v/>
       </c>
     </row>
     <row r="16">
@@ -1465,17 +1509,21 @@
           <t>opus</t>
         </is>
       </c>
-      <c r="E16" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="F16" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" s="4" t="n">
-        <v>0</v>
+      <c r="E16" s="4">
+        <f>COUNTA('P11'!B8:B200)</f>
+        <v/>
+      </c>
+      <c r="F16" s="4">
+        <f>COUNTIF('P11'!F8:F200,"A_VALIDER")+COUNTIF('P11'!F8:F200,"VALIDE")</f>
+        <v/>
+      </c>
+      <c r="G16" s="6">
+        <f>IF(E16=0,0,F16/E16)</f>
+        <v/>
+      </c>
+      <c r="H16" s="4">
+        <f>COUNTIF('P11'!F8:F200,"BLOQUE")</f>
+        <v/>
       </c>
     </row>
     <row r="17">
@@ -1499,17 +1547,21 @@
           <t>sonnet</t>
         </is>
       </c>
-      <c r="E17" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="F17" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" s="4" t="n">
-        <v>0</v>
+      <c r="E17" s="4">
+        <f>COUNTA('P12'!B8:B200)</f>
+        <v/>
+      </c>
+      <c r="F17" s="4">
+        <f>COUNTIF('P12'!F8:F200,"A_VALIDER")+COUNTIF('P12'!F8:F200,"VALIDE")</f>
+        <v/>
+      </c>
+      <c r="G17" s="6">
+        <f>IF(E17=0,0,F17/E17)</f>
+        <v/>
+      </c>
+      <c r="H17" s="4">
+        <f>COUNTIF('P12'!F8:F200,"BLOQUE")</f>
+        <v/>
       </c>
     </row>
     <row r="18">
@@ -1533,17 +1585,21 @@
           <t>sonnet</t>
         </is>
       </c>
-      <c r="E18" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="F18" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G18" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" s="4" t="n">
-        <v>0</v>
+      <c r="E18" s="4">
+        <f>COUNTA('P13'!B8:B200)</f>
+        <v/>
+      </c>
+      <c r="F18" s="4">
+        <f>COUNTIF('P13'!F8:F200,"A_VALIDER")+COUNTIF('P13'!F8:F200,"VALIDE")</f>
+        <v/>
+      </c>
+      <c r="G18" s="6">
+        <f>IF(E18=0,0,F18/E18)</f>
+        <v/>
+      </c>
+      <c r="H18" s="4">
+        <f>COUNTIF('P13'!F8:F200,"BLOQUE")</f>
+        <v/>
       </c>
     </row>
     <row r="19">
@@ -1567,17 +1623,21 @@
           <t>sonnet</t>
         </is>
       </c>
-      <c r="E19" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="F19" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" s="4" t="n">
-        <v>0</v>
+      <c r="E19" s="4">
+        <f>COUNTA('P14'!B8:B200)</f>
+        <v/>
+      </c>
+      <c r="F19" s="4">
+        <f>COUNTIF('P14'!F8:F200,"A_VALIDER")+COUNTIF('P14'!F8:F200,"VALIDE")</f>
+        <v/>
+      </c>
+      <c r="G19" s="6">
+        <f>IF(E19=0,0,F19/E19)</f>
+        <v/>
+      </c>
+      <c r="H19" s="4">
+        <f>COUNTIF('P14'!F8:F200,"BLOQUE")</f>
+        <v/>
       </c>
     </row>
     <row r="20">
@@ -1601,17 +1661,21 @@
           <t>sonnet</t>
         </is>
       </c>
-      <c r="E20" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="F20" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G20" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H20" s="4" t="n">
-        <v>0</v>
+      <c r="E20" s="4">
+        <f>COUNTA('P15'!B8:B200)</f>
+        <v/>
+      </c>
+      <c r="F20" s="4">
+        <f>COUNTIF('P15'!F8:F200,"A_VALIDER")+COUNTIF('P15'!F8:F200,"VALIDE")</f>
+        <v/>
+      </c>
+      <c r="G20" s="6">
+        <f>IF(E20=0,0,F20/E20)</f>
+        <v/>
+      </c>
+      <c r="H20" s="4">
+        <f>COUNTIF('P15'!F8:F200,"BLOQUE")</f>
+        <v/>
       </c>
     </row>
     <row r="21">
@@ -1635,17 +1699,21 @@
           <t>sonnet</t>
         </is>
       </c>
-      <c r="E21" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="F21" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G21" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H21" s="4" t="n">
-        <v>0</v>
+      <c r="E21" s="4">
+        <f>COUNTA('P16'!B8:B200)</f>
+        <v/>
+      </c>
+      <c r="F21" s="4">
+        <f>COUNTIF('P16'!F8:F200,"A_VALIDER")+COUNTIF('P16'!F8:F200,"VALIDE")</f>
+        <v/>
+      </c>
+      <c r="G21" s="6">
+        <f>IF(E21=0,0,F21/E21)</f>
+        <v/>
+      </c>
+      <c r="H21" s="4">
+        <f>COUNTIF('P16'!F8:F200,"BLOQUE")</f>
+        <v/>
       </c>
     </row>
     <row r="22">
@@ -1669,17 +1737,21 @@
           <t>sonnet</t>
         </is>
       </c>
-      <c r="E22" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="F22" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G22" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H22" s="4" t="n">
-        <v>0</v>
+      <c r="E22" s="4">
+        <f>COUNTA('P17'!B8:B200)</f>
+        <v/>
+      </c>
+      <c r="F22" s="4">
+        <f>COUNTIF('P17'!F8:F200,"A_VALIDER")+COUNTIF('P17'!F8:F200,"VALIDE")</f>
+        <v/>
+      </c>
+      <c r="G22" s="6">
+        <f>IF(E22=0,0,F22/E22)</f>
+        <v/>
+      </c>
+      <c r="H22" s="4">
+        <f>COUNTIF('P17'!F8:F200,"BLOQUE")</f>
+        <v/>
       </c>
     </row>
     <row r="23">
@@ -1703,17 +1775,21 @@
           <t>opus</t>
         </is>
       </c>
-      <c r="E23" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="F23" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G23" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H23" s="4" t="n">
-        <v>0</v>
+      <c r="E23" s="4">
+        <f>COUNTA('P18'!B8:B200)</f>
+        <v/>
+      </c>
+      <c r="F23" s="4">
+        <f>COUNTIF('P18'!F8:F200,"A_VALIDER")+COUNTIF('P18'!F8:F200,"VALIDE")</f>
+        <v/>
+      </c>
+      <c r="G23" s="6">
+        <f>IF(E23=0,0,F23/E23)</f>
+        <v/>
+      </c>
+      <c r="H23" s="4">
+        <f>COUNTIF('P18'!F8:F200,"BLOQUE")</f>
+        <v/>
       </c>
     </row>
     <row r="24">
@@ -1737,17 +1813,21 @@
           <t>sonnet</t>
         </is>
       </c>
-      <c r="E24" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="F24" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G24" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H24" s="4" t="n">
-        <v>0</v>
+      <c r="E24" s="4">
+        <f>COUNTA('P19'!B8:B200)</f>
+        <v/>
+      </c>
+      <c r="F24" s="4">
+        <f>COUNTIF('P19'!F8:F200,"A_VALIDER")+COUNTIF('P19'!F8:F200,"VALIDE")</f>
+        <v/>
+      </c>
+      <c r="G24" s="6">
+        <f>IF(E24=0,0,F24/E24)</f>
+        <v/>
+      </c>
+      <c r="H24" s="4">
+        <f>COUNTIF('P19'!F8:F200,"BLOQUE")</f>
+        <v/>
       </c>
     </row>
     <row r="25">
@@ -1756,17 +1836,21 @@
           <t>Total</t>
         </is>
       </c>
-      <c r="E25" s="8" t="n">
-        <v>148</v>
-      </c>
-      <c r="F25" s="8" t="n">
-        <v>31</v>
-      </c>
-      <c r="G25" s="9" t="n">
-        <v>0.2094594594594595</v>
-      </c>
-      <c r="H25" s="8" t="n">
-        <v>0</v>
+      <c r="E25" s="8">
+        <f>SUM(E5:E24)</f>
+        <v/>
+      </c>
+      <c r="F25" s="8">
+        <f>SUM(F5:F24)</f>
+        <v/>
+      </c>
+      <c r="G25" s="9">
+        <f>IF(E25=0,0,F25/E25)</f>
+        <v/>
+      </c>
+      <c r="H25" s="8">
+        <f>SUM(H5:H24)</f>
+        <v/>
       </c>
     </row>
     <row r="27">
@@ -1857,7 +1941,7 @@
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr"/>
@@ -1896,14 +1980,10 @@
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
-        </is>
-      </c>
-      <c r="I30" s="5" t="inlineStr">
-        <is>
-          <t>H-015</t>
-        </is>
-      </c>
+          <t>NON_FAIT</t>
+        </is>
+      </c>
+      <c r="I30" s="5" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
@@ -1939,14 +2019,10 @@
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
-        </is>
-      </c>
-      <c r="I31" s="5" t="inlineStr">
-        <is>
-          <t>H-016</t>
-        </is>
-      </c>
+          <t>NON_FAIT</t>
+        </is>
+      </c>
+      <c r="I31" s="5" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
@@ -1982,14 +2058,10 @@
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
-        </is>
-      </c>
-      <c r="I32" s="5" t="inlineStr">
-        <is>
-          <t>H-017</t>
-        </is>
-      </c>
+          <t>NON_FAIT</t>
+        </is>
+      </c>
+      <c r="I32" s="5" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
@@ -2025,7 +2097,7 @@
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
+          <t>NON_FAIT</t>
         </is>
       </c>
       <c r="I33" s="5" t="inlineStr"/>
@@ -2064,12 +2136,12 @@
       </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
+          <t>NON_FAIT</t>
         </is>
       </c>
       <c r="I34" s="5" t="inlineStr">
         <is>
-          <t>H-003, H-018</t>
+          <t>H-003</t>
         </is>
       </c>
     </row>
@@ -2107,7 +2179,7 @@
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
+          <t>NON_FAIT</t>
         </is>
       </c>
       <c r="I35" s="5" t="inlineStr"/>
@@ -2146,14 +2218,10 @@
       </c>
       <c r="H36" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
-        </is>
-      </c>
-      <c r="I36" s="5" t="inlineStr">
-        <is>
-          <t>H-019</t>
-        </is>
-      </c>
+          <t>NON_FAIT</t>
+        </is>
+      </c>
+      <c r="I36" s="5" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="4" t="n">
@@ -2189,14 +2257,10 @@
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
-        </is>
-      </c>
-      <c r="I37" s="5" t="inlineStr">
-        <is>
-          <t>H-020</t>
-        </is>
-      </c>
+          <t>NON_FAIT</t>
+        </is>
+      </c>
+      <c r="I37" s="5" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="n">
@@ -2232,14 +2296,10 @@
       </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
-        </is>
-      </c>
-      <c r="I38" s="5" t="inlineStr">
-        <is>
-          <t>H-021</t>
-        </is>
-      </c>
+          <t>NON_FAIT</t>
+        </is>
+      </c>
+      <c r="I38" s="5" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="n">
@@ -2275,14 +2335,10 @@
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
-        </is>
-      </c>
-      <c r="I39" s="5" t="inlineStr">
-        <is>
-          <t>H-022</t>
-        </is>
-      </c>
+          <t>NON_FAIT</t>
+        </is>
+      </c>
+      <c r="I39" s="5" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="n">
@@ -2318,14 +2374,10 @@
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
-        </is>
-      </c>
-      <c r="I40" s="5" t="inlineStr">
-        <is>
-          <t>H-023</t>
-        </is>
-      </c>
+          <t>NON_FAIT</t>
+        </is>
+      </c>
+      <c r="I40" s="5" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="n">
@@ -2361,14 +2413,10 @@
       </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
-        </is>
-      </c>
-      <c r="I41" s="5" t="inlineStr">
-        <is>
-          <t>H-024</t>
-        </is>
-      </c>
+          <t>NON_FAIT</t>
+        </is>
+      </c>
+      <c r="I41" s="5" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="4" t="n">
@@ -2404,14 +2452,10 @@
       </c>
       <c r="H42" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
-        </is>
-      </c>
-      <c r="I42" s="5" t="inlineStr">
-        <is>
-          <t>H-025</t>
-        </is>
-      </c>
+          <t>NON_FAIT</t>
+        </is>
+      </c>
+      <c r="I42" s="5" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="n">
@@ -2447,12 +2491,12 @@
       </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
+          <t>NON_FAIT</t>
         </is>
       </c>
       <c r="I43" s="5" t="inlineStr">
         <is>
-          <t>H-004, H-026</t>
+          <t>H-004</t>
         </is>
       </c>
     </row>
@@ -2490,14 +2534,10 @@
       </c>
       <c r="H44" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
-        </is>
-      </c>
-      <c r="I44" s="5" t="inlineStr">
-        <is>
-          <t>H-027</t>
-        </is>
-      </c>
+          <t>NON_FAIT</t>
+        </is>
+      </c>
+      <c r="I44" s="5" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="n">
@@ -2533,14 +2573,10 @@
       </c>
       <c r="H45" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
-        </is>
-      </c>
-      <c r="I45" s="5" t="inlineStr">
-        <is>
-          <t>H-028</t>
-        </is>
-      </c>
+          <t>NON_FAIT</t>
+        </is>
+      </c>
+      <c r="I45" s="5" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="4" t="n">
@@ -2576,14 +2612,10 @@
       </c>
       <c r="H46" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
-        </is>
-      </c>
-      <c r="I46" s="5" t="inlineStr">
-        <is>
-          <t>H-029</t>
-        </is>
-      </c>
+          <t>NON_FAIT</t>
+        </is>
+      </c>
+      <c r="I46" s="5" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="4" t="n">
@@ -2619,12 +2651,12 @@
       </c>
       <c r="H47" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
+          <t>NON_FAIT</t>
         </is>
       </c>
       <c r="I47" s="5" t="inlineStr">
         <is>
-          <t>H-014, H-030</t>
+          <t>H-014</t>
         </is>
       </c>
     </row>
@@ -2662,14 +2694,10 @@
       </c>
       <c r="H48" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
-        </is>
-      </c>
-      <c r="I48" s="5" t="inlineStr">
-        <is>
-          <t>H-031</t>
-        </is>
-      </c>
+          <t>NON_FAIT</t>
+        </is>
+      </c>
+      <c r="I48" s="5" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="4" t="n">
@@ -2705,7 +2733,7 @@
       </c>
       <c r="H49" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
+          <t>NON_FAIT</t>
         </is>
       </c>
       <c r="I49" s="5" t="inlineStr"/>
@@ -2744,7 +2772,7 @@
       </c>
       <c r="H50" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
+          <t>NON_FAIT</t>
         </is>
       </c>
       <c r="I50" s="5" t="inlineStr"/>
@@ -2783,14 +2811,10 @@
       </c>
       <c r="H51" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
-        </is>
-      </c>
-      <c r="I51" s="5" t="inlineStr">
-        <is>
-          <t>H-032</t>
-        </is>
-      </c>
+          <t>NON_FAIT</t>
+        </is>
+      </c>
+      <c r="I51" s="5" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="4" t="n">
@@ -2826,14 +2850,10 @@
       </c>
       <c r="H52" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
-        </is>
-      </c>
-      <c r="I52" s="5" t="inlineStr">
-        <is>
-          <t>H-033</t>
-        </is>
-      </c>
+          <t>NON_FAIT</t>
+        </is>
+      </c>
+      <c r="I52" s="5" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="4" t="n">
@@ -2869,14 +2889,10 @@
       </c>
       <c r="H53" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
-        </is>
-      </c>
-      <c r="I53" s="5" t="inlineStr">
-        <is>
-          <t>H-034</t>
-        </is>
-      </c>
+          <t>NON_FAIT</t>
+        </is>
+      </c>
+      <c r="I53" s="5" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="4" t="n">
@@ -2912,14 +2928,10 @@
       </c>
       <c r="H54" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
-        </is>
-      </c>
-      <c r="I54" s="5" t="inlineStr">
-        <is>
-          <t>H-035</t>
-        </is>
-      </c>
+          <t>NON_FAIT</t>
+        </is>
+      </c>
+      <c r="I54" s="5" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="4" t="n">
@@ -2927,7 +2939,7 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>P3 · Conteneurisation et intégration continue GitHub Actions</t>
+          <t>P3 · Conteneurisation et intégration continue GitLab</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
@@ -2955,7 +2967,7 @@
       </c>
       <c r="H55" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
+          <t>NON_FAIT</t>
         </is>
       </c>
       <c r="I55" s="5" t="inlineStr">
@@ -2970,7 +2982,7 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>P3 · Conteneurisation et intégration continue GitHub Actions</t>
+          <t>P3 · Conteneurisation et intégration continue GitLab</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
@@ -2998,14 +3010,10 @@
       </c>
       <c r="H56" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
-        </is>
-      </c>
-      <c r="I56" s="5" t="inlineStr">
-        <is>
-          <t>H-036</t>
-        </is>
-      </c>
+          <t>NON_FAIT</t>
+        </is>
+      </c>
+      <c r="I56" s="5" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="4" t="n">
@@ -3013,7 +3021,7 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>P3 · Conteneurisation et intégration continue GitHub Actions</t>
+          <t>P3 · Conteneurisation et intégration continue GitLab</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
@@ -3041,7 +3049,7 @@
       </c>
       <c r="H57" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
+          <t>NON_FAIT</t>
         </is>
       </c>
       <c r="I57" s="5" t="inlineStr"/>
@@ -3052,7 +3060,7 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>P3 · Conteneurisation et intégration continue GitHub Actions</t>
+          <t>P3 · Conteneurisation et intégration continue GitLab</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
@@ -3062,7 +3070,7 @@
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>Workflow GitHub Actions</t>
+          <t>Pipeline .gitlab-ci.yml</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
@@ -3080,12 +3088,12 @@
       </c>
       <c r="H58" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
+          <t>NON_FAIT</t>
         </is>
       </c>
       <c r="I58" s="5" t="inlineStr">
         <is>
-          <t>H-002, H-037</t>
+          <t>H-002</t>
         </is>
       </c>
     </row>
@@ -3095,7 +3103,7 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>P3 · Conteneurisation et intégration continue GitHub Actions</t>
+          <t>P3 · Conteneurisation et intégration continue GitLab</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
@@ -3123,7 +3131,7 @@
       </c>
       <c r="H59" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
+          <t>NON_FAIT</t>
         </is>
       </c>
       <c r="I59" s="5" t="inlineStr"/>
@@ -8044,8 +8052,9 @@
           <t>Avancement</t>
         </is>
       </c>
-      <c r="B5" s="12" t="n">
-        <v>0</v>
+      <c r="B5" s="12">
+        <f>IF(COUNTA(B8:B200)=0,0,(COUNTIF(F8:F200,"A_VALIDER")+COUNTIF(F8:F200,"VALIDE"))/COUNTA(B8:B200))</f>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -8607,8 +8616,9 @@
           <t>Avancement</t>
         </is>
       </c>
-      <c r="B5" s="12" t="n">
-        <v>0</v>
+      <c r="B5" s="12">
+        <f>IF(COUNTA(B8:B200)=0,0,(COUNTIF(F8:F200,"A_VALIDER")+COUNTIF(F8:F200,"VALIDE"))/COUNTA(B8:B200))</f>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -9043,8 +9053,9 @@
           <t>Avancement</t>
         </is>
       </c>
-      <c r="B5" s="12" t="n">
-        <v>0</v>
+      <c r="B5" s="12">
+        <f>IF(COUNTA(B8:B200)=0,0,(COUNTIF(F8:F200,"A_VALIDER")+COUNTIF(F8:F200,"VALIDE"))/COUNTA(B8:B200))</f>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -9651,8 +9662,9 @@
           <t>Avancement</t>
         </is>
       </c>
-      <c r="B5" s="12" t="n">
-        <v>0</v>
+      <c r="B5" s="12">
+        <f>IF(COUNTA(B8:B200)=0,0,(COUNTIF(F8:F200,"A_VALIDER")+COUNTIF(F8:F200,"VALIDE"))/COUNTA(B8:B200))</f>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -10167,8 +10179,9 @@
           <t>Avancement</t>
         </is>
       </c>
-      <c r="B5" s="12" t="n">
-        <v>0</v>
+      <c r="B5" s="12">
+        <f>IF(COUNTA(B8:B200)=0,0,(COUNTIF(F8:F200,"A_VALIDER")+COUNTIF(F8:F200,"VALIDE"))/COUNTA(B8:B200))</f>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -10645,8 +10658,9 @@
           <t>Avancement</t>
         </is>
       </c>
-      <c r="B5" s="12" t="n">
-        <v>0</v>
+      <c r="B5" s="12">
+        <f>IF(COUNTA(B8:B200)=0,0,(COUNTIF(F8:F200,"A_VALIDER")+COUNTIF(F8:F200,"VALIDE"))/COUNTA(B8:B200))</f>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -11077,8 +11091,9 @@
           <t>Avancement</t>
         </is>
       </c>
-      <c r="B5" s="12" t="n">
-        <v>0</v>
+      <c r="B5" s="12">
+        <f>IF(COUNTA(B8:B200)=0,0,(COUNTIF(F8:F200,"A_VALIDER")+COUNTIF(F8:F200,"VALIDE"))/COUNTA(B8:B200))</f>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -11551,8 +11566,9 @@
           <t>Avancement</t>
         </is>
       </c>
-      <c r="B5" s="12" t="n">
-        <v>0</v>
+      <c r="B5" s="12">
+        <f>IF(COUNTA(B8:B200)=0,0,(COUNTIF(F8:F200,"A_VALIDER")+COUNTIF(F8:F200,"VALIDE"))/COUNTA(B8:B200))</f>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -12029,8 +12045,9 @@
           <t>Avancement</t>
         </is>
       </c>
-      <c r="B5" s="12" t="n">
-        <v>0</v>
+      <c r="B5" s="12">
+        <f>IF(COUNTA(B8:B200)=0,0,(COUNTIF(F8:F200,"A_VALIDER")+COUNTIF(F8:F200,"VALIDE"))/COUNTA(B8:B200))</f>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -12503,8 +12520,9 @@
           <t>Avancement</t>
         </is>
       </c>
-      <c r="B5" s="12" t="n">
-        <v>0</v>
+      <c r="B5" s="12">
+        <f>IF(COUNTA(B8:B200)=0,0,(COUNTIF(F8:F200,"A_VALIDER")+COUNTIF(F8:F200,"VALIDE"))/COUNTA(B8:B200))</f>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -13039,7 +13057,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>VALIDEE</t>
+          <t>EN_COURS</t>
         </is>
       </c>
     </row>
@@ -13061,8 +13079,9 @@
           <t>Avancement</t>
         </is>
       </c>
-      <c r="B5" s="12" t="n">
-        <v>1</v>
+      <c r="B5" s="12">
+        <f>IF(COUNTA(B8:B200)=0,0,(COUNTIF(F8:F200,"A_VALIDER")+COUNTIF(F8:F200,"VALIDE"))/COUNTA(B8:B200))</f>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -13150,7 +13169,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
+          <t>EN_COURS</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
@@ -13192,7 +13211,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
+          <t>NON_FAIT</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
@@ -13206,11 +13225,7 @@
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr"/>
-      <c r="J9" s="5" t="inlineStr">
-        <is>
-          <t>H-015 (OUVERTE)</t>
-        </is>
-      </c>
+      <c r="J9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
@@ -13238,7 +13253,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
+          <t>NON_FAIT</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
@@ -13252,11 +13267,7 @@
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr"/>
-      <c r="J10" s="5" t="inlineStr">
-        <is>
-          <t>H-016 (OUVERTE)</t>
-        </is>
-      </c>
+      <c r="J10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
@@ -13284,7 +13295,7 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
+          <t>NON_FAIT</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
@@ -13298,11 +13309,7 @@
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr"/>
-      <c r="J11" s="5" t="inlineStr">
-        <is>
-          <t>H-017 (REPONDUE)</t>
-        </is>
-      </c>
+      <c r="J11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
@@ -13330,7 +13337,7 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
+          <t>NON_FAIT</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
@@ -13372,7 +13379,7 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
+          <t>NON_FAIT</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
@@ -13388,8 +13395,7 @@
       <c r="I13" s="5" t="inlineStr"/>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>H-003 (REPONDUE)
-H-018 (OUVERTE)</t>
+          <t>H-003 (REPONDUE)</t>
         </is>
       </c>
     </row>
@@ -13552,8 +13558,9 @@
           <t>Avancement</t>
         </is>
       </c>
-      <c r="B5" s="12" t="n">
-        <v>0</v>
+      <c r="B5" s="12">
+        <f>IF(COUNTA(B8:B200)=0,0,(COUNTIF(F8:F200,"A_VALIDER")+COUNTIF(F8:F200,"VALIDE"))/COUNTA(B8:B200))</f>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -14072,8 +14079,9 @@
           <t>Avancement</t>
         </is>
       </c>
-      <c r="B5" s="12" t="n">
-        <v>0</v>
+      <c r="B5" s="12">
+        <f>IF(COUNTA(B8:B200)=0,0,(COUNTIF(F8:F200,"A_VALIDER")+COUNTIF(F8:F200,"VALIDE"))/COUNTA(B8:B200))</f>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -14487,7 +14495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I41"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -14622,7 +14630,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>REPONDUE</t>
+          <t>OUVERTE</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -14652,7 +14660,7 @@
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>48) : Choix utilisateur (2026-10-16) : le dépôt du projet est sur GitHub (hajar-hamid-coder/gprojet, public) ; l'intégration continue se fait avec GitHub Actions et l'image est publiée sur ghcr.io. GitLab reste une intégration fonctionnelle de la plateforme (P12-P13).</t>
+          <t>en attente</t>
         </is>
       </c>
     </row>
@@ -15220,1089 +15228,8 @@
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>H-015</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>P0-T02</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>OUVERTE</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-16 11:51</t>
-        </is>
-      </c>
-      <c r="F19" s="5" t="inlineStr">
-        <is>
-          <t>Que faire si PG_BIN pointe vers un dossier sans binaires PostgreSQL ?</t>
-        </is>
-      </c>
-      <c r="G19" s="5" t="inlineStr">
-        <is>
-          <t>PG_BIN est exclusif dans verifier-env.py (pas de repli), sinon le cas test PG_BIN vide ne peut jamais sortir en 1 ici</t>
-        </is>
-      </c>
-      <c r="H19" s="5" t="inlineStr">
-        <is>
-          <t>pg-test.py retombe sur les chemins par défaut : comportement différent entre les deux scripts</t>
-        </is>
-      </c>
-      <c r="I19" s="5" t="inlineStr">
-        <is>
-          <t>en attente</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>H-016</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>P0-T03</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>OUVERTE</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-16 11:52</t>
-        </is>
-      </c>
-      <c r="F20" s="5" t="inlineStr">
-        <is>
-          <t>database/03-tests-integrite.sql compte-t-il 13 blocs ERREUR + 5 OK comme l'indique la tâche ?</t>
-        </is>
-      </c>
-      <c r="G20" s="5" t="inlineStr">
-        <is>
-          <t>Il contient 12 ERREUR + 6 OK (total 18 conforme) ; la répartition 13+5 est une erreur de décompte, seul le total compte</t>
-        </is>
-      </c>
-      <c r="H20" s="5" t="inlineStr">
-        <is>
-          <t>Si faux, un bloc attendu ERREUR manquerait dans le fichier 03</t>
-        </is>
-      </c>
-      <c r="I20" s="5" t="inlineStr">
-        <is>
-          <t>en attente</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>H-017</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>P0-T04</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>REPONDUE</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-16 11:55</t>
-        </is>
-      </c>
-      <c r="F21" s="5" t="inlineStr">
-        <is>
-          <t>FluentAssertions 8.x (licence commerciale Xceed) est-il acceptable pour un projet d'État ?</t>
-        </is>
-      </c>
-      <c r="G21" s="5" t="inlineStr">
-        <is>
-          <t>Version 8.11.0 retenue pour l'instant ; si la licence pose problème, épingler 7.x (Apache 2.0) dans Directory.Packages.props</t>
-        </is>
-      </c>
-      <c r="H21" s="5" t="inlineStr">
-        <is>
-          <t>Aucun avant l'écriture des premiers tests (P0-T05+ ou P1)</t>
-        </is>
-      </c>
-      <c r="I21" s="5" t="inlineStr">
-        <is>
-          <t>51) : Non : épingler FluentAssertions 7.x (Apache 2.0), pas de licence commerciale</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>H-018</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>P0-T06</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>OUVERTE</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-16 11:58</t>
-        </is>
-      </c>
-      <c r="F22" s="5" t="inlineStr">
-        <is>
-          <t>graphify (CLI, paquet PyPI graphifyy) est absent du poste et uv (requis pour l'installer) est absent aussi : faut-il les installer maintenant pour le graphe de connaissances du code ?</t>
-        </is>
-      </c>
-      <c r="G22" s="5" t="inlineStr">
-        <is>
-          <t>Ne pas installer maintenant : graphify n'est utile qu'à partir de la première phase qui produit du code (P1). Installation prévue via scripts/installer-outils.ps1 (étapes uv puis uv tool install graphifyy, puis graphify install --project) avant P1 ; en attendant, la recherche se fait par Grep/Explore.</t>
-        </is>
-      </c>
-      <c r="H22" s="5" t="inlineStr">
-        <is>
-          <t>Sans graphify, les requêtes 'graphify query' de CLAUDE.md ne fonctionnent pas : le repérage du code se fait par recherche classique (plus lent, plus de tokens). Aucun blocage de P0.</t>
-        </is>
-      </c>
-      <c r="I22" s="5" t="inlineStr">
-        <is>
-          <t>en attente</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>H-019</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>P1-T02</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>OUVERTE</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-16 13:01</t>
-        </is>
-      </c>
-      <c r="F23" s="5" t="inlineStr">
-        <is>
-          <t>Comment reconnaître un contrôleur, et la liste blanche System.* de Contracts suffit-elle ?</t>
-        </is>
-      </c>
-      <c r="G23" s="5" t="inlineStr">
-        <is>
-          <t>Contrôleur = hérite de ControllerBase ou nom en *Controller ; Contracts autorise tout System.* (les API absentes du navigateur ne sont pas détectées, la compilation du front en P2 servira de seconde garde)</t>
-        </is>
-      </c>
-      <c r="H23" s="5" t="inlineStr">
-        <is>
-          <t>Des endpoints minimal API échapperaient à la règle ; une API System non disponible en WASM serait détectée seulement à la compilation du front</t>
-        </is>
-      </c>
-      <c r="I23" s="5" t="inlineStr">
-        <is>
-          <t>en attente</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>H-020</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>P1-T03</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>OUVERTE</t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-16 13:05</t>
-        </is>
-      </c>
-      <c r="F24" s="5" t="inlineStr">
-        <is>
-          <t>Dans quel fuseau calcule-t-on la date du jour (saisie des temps, échéances) ?</t>
-        </is>
-      </c>
-      <c r="G24" s="5" t="inlineStr">
-        <is>
-          <t>Fuseau Africa/Casablanca (HCP) ; IHorloge.Aujourdhui est calculé dans ce fuseau, Maintenant reste en UTC</t>
-        </is>
-      </c>
-      <c r="H24" s="5" t="inlineStr">
-        <is>
-          <t>Si un autre fuseau est attendu, changer la valeur passée à HorlogeSysteme ; en UTC pur, les saisies entre minuit et 1 h seraient datées de la veille</t>
-        </is>
-      </c>
-      <c r="I24" s="5" t="inlineStr">
-        <is>
-          <t>en attente</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>H-021</t>
-        </is>
-      </c>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>P1-T04</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>OUVERTE</t>
-        </is>
-      </c>
-      <c r="D25" s="4" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-16 13:15</t>
-        </is>
-      </c>
-      <c r="F25" s="5" t="inlineStr">
-        <is>
-          <t>patte.card_min (CHECK IN numérique 0,1) et correspondance_type.type_logique (sans CHECK) doivent-ils devenir des énumérations ?</t>
-        </is>
-      </c>
-      <c r="G25" s="5" t="inlineStr">
-        <is>
-          <t>Non : card_min reste short, correspondance_type.type_logique reste string ; seuls les CHECK IN à valeurs texte deviennent des enums (49 enums, 54 contraintes contrôlées)</t>
-        </is>
-      </c>
-      <c r="H25" s="5" t="inlineStr">
-        <is>
-          <t>Si faux : créer CardinaliteMin et/ou ajouter le CHECK au SQL puis typer en TypeLogique</t>
-        </is>
-      </c>
-      <c r="I25" s="5" t="inlineStr">
-        <is>
-          <t>en attente</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>H-022</t>
-        </is>
-      </c>
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>P1-T05</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t>OUVERTE</t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="E26" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-16 13:27</t>
-        </is>
-      </c>
-      <c r="F26" s="5" t="inlineStr">
-        <is>
-          <t>Comment reproduire l'index sur expression ux_agent_email (lower(email)) et le trigger de lecture seule de commun.historique, non modélisables par EF ?</t>
-        </is>
-      </c>
-      <c r="G26" s="5" t="inlineStr">
-        <is>
-          <t>Le modèle EF déclare ux_agent_email sur email (shortcut commenté) ; la migration initiale P1-T06 recrée l'index sur lower(email) et le trigger tg_historique_lecture_seule en SQL brut</t>
-        </is>
-      </c>
-      <c r="H26" s="5" t="inlineStr">
-        <is>
-          <t>Si oublié en P1-T06 : unicité de l'email sensible à la casse et journal d'historique modifiable</t>
-        </is>
-      </c>
-      <c r="I26" s="5" t="inlineStr">
-        <is>
-          <t>en attente</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>H-023</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>P1-T06</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>OUVERTE</t>
-        </is>
-      </c>
-      <c r="D27" s="4" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="E27" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-16 14:45</t>
-        </is>
-      </c>
-      <c r="F27" s="5" t="inlineStr">
-        <is>
-          <t>La comparaison de schéma doit-elle couvrir l'ordre des colonnes et le contenu des données de référence ?</t>
-        </is>
-      </c>
-      <c r="G27" s="5" t="inlineStr">
-        <is>
-          <t>Non : type, nullabilité, défaut, contraintes, index, triggers, fonctions et nombre de lignes par table suffisent ; les données sont une copie figée de 02 embarquée dans la migration</t>
-        </is>
-      </c>
-      <c r="H27" s="5" t="inlineStr">
-        <is>
-          <t>Une différence d'ordre de colonnes ou de valeurs (même nombre de lignes) ne serait pas détectée</t>
-        </is>
-      </c>
-      <c r="I27" s="5" t="inlineStr">
-        <is>
-          <t>en attente</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>H-024</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>P1-T07</t>
-        </is>
-      </c>
-      <c r="C28" s="4" t="inlineStr">
-        <is>
-          <t>OUVERTE</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="E28" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-16 14:49</t>
-        </is>
-      </c>
-      <c r="F28" s="5" t="inlineStr">
-        <is>
-          <t>Quel agent pour les écritures hors requête (jobs, données initiales), et type_cible sans schéma est-il acceptable ?</t>
-        </is>
-      </c>
-      <c r="G28" s="5" t="inlineStr">
-        <is>
-          <t>Un utilisateur système (ICurrentUser dédié) sera fourni pour les traitements hors requête ; type_cible = nom de table sans schéma (unique entre schémas, ≤ 30 caractères)</t>
-        </is>
-      </c>
-      <c r="H28" s="5" t="inlineStr">
-        <is>
-          <t>Sans utilisateur système, cree_par/agent_id seraient vides pour ces écritures ; un futur doublon de nom de table entre schémas rendrait type_cible ambigu</t>
-        </is>
-      </c>
-      <c r="I28" s="5" t="inlineStr">
-        <is>
-          <t>en attente</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>H-025</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>P1-T08</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>OUVERTE</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-16 14:54</t>
-        </is>
-      </c>
-      <c r="F29" s="5" t="inlineStr">
-        <is>
-          <t>Quels repositories d'agrégat livrer dans le socle, et où enregistrer UnitOfWork/repositories dans la DI ?</t>
-        </is>
-      </c>
-      <c r="G29" s="5" t="inlineStr">
-        <is>
-          <t>Un seul repository réel (Compétence) pour démontrer le motif ; les autres arrivent avec leurs modules (P4, P5…). Enregistrement DI dans la tâche de composition (P1-T09/T10)</t>
-        </is>
-      </c>
-      <c r="H29" s="5" t="inlineStr">
-        <is>
-          <t>Effort minime pour changer d'agrégat ; aucun enregistrement DI tant que Program.cs n'est pas composé</t>
-        </is>
-      </c>
-      <c r="I29" s="5" t="inlineStr">
-        <is>
-          <t>en attente</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>H-026</t>
-        </is>
-      </c>
-      <c r="B30" s="4" t="inlineStr">
-        <is>
-          <t>P1-T09</t>
-        </is>
-      </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t>OUVERTE</t>
-        </is>
-      </c>
-      <c r="D30" s="4" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="E30" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-16 15:00</t>
-        </is>
-      </c>
-      <c r="F30" s="5" t="inlineStr">
-        <is>
-          <t>Quel utilisateur courant avant Keycloak (P18), et quel code HTTP pour RegleMetierException ?</t>
-        </is>
-      </c>
-      <c r="G30" s="5" t="inlineStr">
-        <is>
-          <t>ICurrentUser provisoire = agent SYSTEME (Id Guid.Empty, sans rôle), shortcut à remplacer en P18 ; RegleMetierException → 422, validation FluentValidation → 400</t>
-        </is>
-      </c>
-      <c r="H30" s="5" t="inlineStr">
-        <is>
-          <t>cree_par/agent_id valent Guid.Empty jusqu'en P18 (colonnes sans FK) ; changer le code 422 est une ligne dans GestionnaireExceptions</t>
-        </is>
-      </c>
-      <c r="I30" s="5" t="inlineStr">
-        <is>
-          <t>en attente</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>H-027</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>P1-T10</t>
-        </is>
-      </c>
-      <c r="C31" s="4" t="inlineStr">
-        <is>
-          <t>OUVERTE</t>
-        </is>
-      </c>
-      <c r="D31" s="4" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-16 15:11</t>
-        </is>
-      </c>
-      <c r="F31" s="5" t="inlineStr">
-        <is>
-          <t>Quels rôles déduire dans le socle, et comment traiter une délégation révoquée ?</t>
-        </is>
-      </c>
-      <c r="G31" s="5" t="inlineStr">
-        <is>
-          <t>Deux rôles déduits : RESPONSABLE_ENTITE (responsable d'une entité active) et DELEGATAIRE (délégation non supprimée couvrant aujourd'hui) ; révocation = suppression logique ; les rôles Directeur/Chef de division/Chef de service seront déduits du niveau de l'entité dans le module Organisation (P4). Hors requête et en Production avant P18 : utilisateur SYSTEME et 401 sur les contrôleurs</t>
-        </is>
-      </c>
-      <c r="H31" s="5" t="inlineStr">
-        <is>
-          <t>Enrichir DevAuthHandler si d'autres rôles sont requis ; prévoir un agent système en base si cree_par doit référencer un agent réel</t>
-        </is>
-      </c>
-      <c r="I31" s="5" t="inlineStr">
-        <is>
-          <t>en attente</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>H-028</t>
-        </is>
-      </c>
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>P1-T11</t>
-        </is>
-      </c>
-      <c r="C32" s="4" t="inlineStr">
-        <is>
-          <t>OUVERTE</t>
-        </is>
-      </c>
-      <c r="D32" s="4" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="E32" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-16 15:18</t>
-        </is>
-      </c>
-      <c r="F32" s="5" t="inlineStr">
-        <is>
-          <t>Quels jours fériés 2026 retenir pour la démo, notamment les fêtes religieuses mobiles ?</t>
-        </is>
-      </c>
-      <c r="G32" s="5" t="inlineStr">
-        <is>
-          <t>Calendrier civil marocain pour les jours fixes ; fêtes mobiles 2026 à des dates indicatives (marquées « indicatif »), à confirmer par l'annonce officielle</t>
-        </is>
-      </c>
-      <c r="H32" s="5" t="inlineStr">
-        <is>
-          <t>Seules les données de démonstration seraient à corriger ; aucun calcul métier n'est encore branché dessus</t>
-        </is>
-      </c>
-      <c r="I32" s="5" t="inlineStr">
-        <is>
-          <t>en attente</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>H-029</t>
-        </is>
-      </c>
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>P2-T01</t>
-        </is>
-      </c>
-      <c r="C33" s="4" t="inlineStr">
-        <is>
-          <t>OUVERTE</t>
-        </is>
-      </c>
-      <c r="D33" s="4" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="E33" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-16 15:42</t>
-        </is>
-      </c>
-      <c r="F33" s="5" t="inlineStr">
-        <is>
-          <t>Quel premier DTO partagé, et où exposer la santé pour le front ?</t>
-        </is>
-      </c>
-      <c r="G33" s="5" t="inlineStr">
-        <is>
-          <t>SanteDto (record Statut) renvoyé par GET /api/health (minimal API anonyme), consommé par SanteApiClient ; /health et /health/ready restent pour l'exploitation</t>
-        </is>
-      </c>
-      <c r="H33" s="5" t="inlineStr">
-        <is>
-          <t>Renommage ou déplacement minime si un autre DTO de référence est préféré</t>
-        </is>
-      </c>
-      <c r="I33" s="5" t="inlineStr">
-        <is>
-          <t>en attente</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>H-030</t>
-        </is>
-      </c>
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t>P2-T02</t>
-        </is>
-      </c>
-      <c r="C34" s="4" t="inlineStr">
-        <is>
-          <t>OUVERTE</t>
-        </is>
-      </c>
-      <c r="D34" s="4" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="E34" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-16 15:47</t>
-        </is>
-      </c>
-      <c r="F34" s="5" t="inlineStr">
-        <is>
-          <t>Quelles classes de badge de statut prévoir, et comment mapper les statuts configurables de tâche/ticket ?</t>
-        </is>
-      </c>
-      <c r="G34" s="5" t="inlineStr">
-        <is>
-          <t>Classes kebab-case déduites des enums de statut du backend ; les workflows configurables (CategorieStatut) se mappent sur a-faire / en-cours / termine ; d'autres classes s'ajouteront au besoin</t>
-        </is>
-      </c>
-      <c r="H34" s="5" t="inlineStr">
-        <is>
-          <t>Ajout de classes dans app.gp.css si un statut n'est pas couvert</t>
-        </is>
-      </c>
-      <c r="I34" s="5" t="inlineStr">
-        <is>
-          <t>en attente</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>H-031</t>
-        </is>
-      </c>
-      <c r="B35" s="4" t="inlineStr">
-        <is>
-          <t>P2-T03</t>
-        </is>
-      </c>
-      <c r="C35" s="4" t="inlineStr">
-        <is>
-          <t>OUVERTE</t>
-        </is>
-      </c>
-      <c r="D35" s="4" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="E35" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-16 15:52</t>
-        </is>
-      </c>
-      <c r="F35" s="5" t="inlineStr">
-        <is>
-          <t>Qui voit le menu Administration, et quand le rôle DIRECTEUR sera-t-il attribué ?</t>
-        </is>
-      </c>
-      <c r="G35" s="5" t="inlineStr">
-        <is>
-          <t>Administration = DIRECTEUR ou RESPONSABLE_ENTITE ; DIRECTEUR est déclaré (Contracts/Commun/RolesApplication) mais déduit côté serveur seulement en P4 ; libellés en dur en français tant que l'i18n (resx) n'existe pas</t>
-        </is>
-      </c>
-      <c r="H35" s="5" t="inlineStr">
-        <is>
-          <t>Politiques.cs à ajuster si besoin ; « Portefeuille direction » invisible pour tous jusqu'en P4 ; libellés à basculer en resx plus tard</t>
-        </is>
-      </c>
-      <c r="I35" s="5" t="inlineStr">
-        <is>
-          <t>en attente</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="4" t="inlineStr">
-        <is>
-          <t>H-032</t>
-        </is>
-      </c>
-      <c r="B36" s="4" t="inlineStr">
-        <is>
-          <t>P2-T06</t>
-        </is>
-      </c>
-      <c r="C36" s="4" t="inlineStr">
-        <is>
-          <t>OUVERTE</t>
-        </is>
-      </c>
-      <c r="D36" s="4" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="E36" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-16 16:05</t>
-        </is>
-      </c>
-      <c r="F36" s="5" t="inlineStr">
-        <is>
-          <t>Les rôles sont-ils figés dans le cookie, et les pages doivent-elles rediriger les anonymes vers /connexion ?</t>
-        </is>
-      </c>
-      <c r="G36" s="5" t="inlineStr">
-        <is>
-          <t>Rôles lus au login et valables 8 h glissantes (shortcut jusqu'à Keycloak P18) ; pas de redirection automatique vers /connexion dans le socle, les gardes de pages viendront avec les pages métier ; anti-CSRF par en-tête X-CSRF: 1 obligatoire dès qu'un cookie de session est présent</t>
-        </is>
-      </c>
-      <c r="H36" s="5" t="inlineStr">
-        <is>
-          <t>Un changement de rôle ne s'applique qu'à la reconnexion ; ajouter des gardes de pages au besoin</t>
-        </is>
-      </c>
-      <c r="I36" s="5" t="inlineStr">
-        <is>
-          <t>en attente</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="4" t="inlineStr">
-        <is>
-          <t>H-033</t>
-        </is>
-      </c>
-      <c r="B37" s="4" t="inlineStr">
-        <is>
-          <t>P2-T07</t>
-        </is>
-      </c>
-      <c r="C37" s="4" t="inlineStr">
-        <is>
-          <t>OUVERTE</t>
-        </is>
-      </c>
-      <c r="D37" s="4" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="E37" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-16 16:10</t>
-        </is>
-      </c>
-      <c r="F37" s="5" t="inlineStr">
-        <is>
-          <t>D'où viendront le niveau et le chemin du périmètre côté front, et quel délai de disparition des notifications ?</t>
-        </is>
-      </c>
-      <c r="G37" s="5" t="inlineStr">
-        <is>
-          <t>PerimetreState expose Definir(...) ; il sera alimenté par le module Organisation (P4), sans endpoint fantôme maintenant. Notifications : 6 s pour tous les types, réglable</t>
-        </is>
-      </c>
-      <c r="H37" s="5" t="inlineStr">
-        <is>
-          <t>Un endpoint ou un claim supplémentaire en P4 ; réglage simple du délai</t>
-        </is>
-      </c>
-      <c r="I37" s="5" t="inlineStr">
-        <is>
-          <t>en attente</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="4" t="inlineStr">
-        <is>
-          <t>H-034</t>
-        </is>
-      </c>
-      <c r="B38" s="4" t="inlineStr">
-        <is>
-          <t>P2-T08</t>
-        </is>
-      </c>
-      <c r="C38" s="4" t="inlineStr">
-        <is>
-          <t>OUVERTE</t>
-        </is>
-      </c>
-      <c r="D38" s="4" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="E38" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-16 16:22</t>
-        </is>
-      </c>
-      <c r="F38" s="5" t="inlineStr">
-        <is>
-          <t>Culture par défaut, police arabe et relecture des traductions ?</t>
-        </is>
-      </c>
-      <c r="G38" s="5" t="inlineStr">
-        <is>
-          <t>fr-MA par défaut (repli), en et ar-MA ; arabe affiché avec la pile système (Geist sans glyphes arabes, aucune police téléchargée) ; traductions en/ar rédigées sans relecture native</t>
-        </is>
-      </c>
-      <c r="H38" s="5" t="inlineStr">
-        <is>
-          <t>Changer Langues.Defaut ; ajouter une police arabe auto-hébergée si le rendu système déplaît ; faire relire en et ar avant la mise en production</t>
-        </is>
-      </c>
-      <c r="I38" s="5" t="inlineStr">
-        <is>
-          <t>en attente</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="4" t="inlineStr">
-        <is>
-          <t>H-035</t>
-        </is>
-      </c>
-      <c r="B39" s="4" t="inlineStr">
-        <is>
-          <t>P2-T09</t>
-        </is>
-      </c>
-      <c r="C39" s="4" t="inlineStr">
-        <is>
-          <t>OUVERTE</t>
-        </is>
-      </c>
-      <c r="D39" s="4" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="E39" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-16 16:26</t>
-        </is>
-      </c>
-      <c r="F39" s="5" t="inlineStr">
-        <is>
-          <t>Faut-il brancher dès maintenant la page Erreur sur un ErrorBoundary et Accès refusé sur une garde de routes ?</t>
-        </is>
-      </c>
-      <c r="G39" s="5" t="inlineStr">
-        <is>
-          <t>Non : pages prêtes mais non câblées (pas d'AuthorizeRouteView ni d'ErrorBoundary) jusqu'aux pages métier ; textes de chargement initial et d'erreur fatale de index.html en français (hors localizer)</t>
-        </is>
-      </c>
-      <c r="H39" s="5" t="inlineStr">
-        <is>
-          <t>Câblage à ajouter avec les premières pages protégées ; en/ar voient deux textes français pendant le chargement</t>
-        </is>
-      </c>
-      <c r="I39" s="5" t="inlineStr">
-        <is>
-          <t>en attente</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="4" t="inlineStr">
-        <is>
-          <t>H-036</t>
-        </is>
-      </c>
-      <c r="B40" s="4" t="inlineStr">
-        <is>
-          <t>P3-T02</t>
-        </is>
-      </c>
-      <c r="C40" s="4" t="inlineStr">
-        <is>
-          <t>OUVERTE</t>
-        </is>
-      </c>
-      <c r="D40" s="4" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="E40" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-21 11:03</t>
-        </is>
-      </c>
-      <c r="F40" s="5" t="inlineStr">
-        <is>
-          <t>Le port 8080 du poste est occupé par un conteneur youtrack étranger au projet : faut-il changer le port par défaut de l'app dans le compose ?</t>
-        </is>
-      </c>
-      <c r="G40" s="5" t="inlineStr">
-        <is>
-          <t>Port par défaut 8080 conservé, surchargeable par APP_HOST_PORT dans deploy/.env ; tests faits sur 18080 sans arrêter youtrack.</t>
-        </is>
-      </c>
-      <c r="H40" s="5" t="inlineStr">
-        <is>
-          <t>Avec youtrack actif, http://localhost:8080 répond YouTrack et non GestionProjet tant que APP_HOST_PORT n'est pas défini.</t>
-        </is>
-      </c>
-      <c r="I40" s="5" t="inlineStr">
-        <is>
-          <t>en attente</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="4" t="inlineStr">
-        <is>
-          <t>H-037</t>
-        </is>
-      </c>
-      <c r="B41" s="4" t="inlineStr">
-        <is>
-          <t>P3-T04</t>
-        </is>
-      </c>
-      <c r="C41" s="4" t="inlineStr">
-        <is>
-          <t>OUVERTE</t>
-        </is>
-      </c>
-      <c r="D41" s="4" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="E41" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-21 11:16</t>
-        </is>
-      </c>
-      <c r="F41" s="5" t="inlineStr">
-        <is>
-          <t>Les versions d'actions épinglées et le comportement réel du workflow (Trivy bloquant sur CRITICAL/HIGH, environnement production) ne peuvent être constatés qu'après le push : faut-il assouplir Trivy ?</t>
-        </is>
-      </c>
-      <c r="G41" s="5" t="inlineStr">
-        <is>
-          <t>Trivy bloquant (exit-code 1, CRITICAL/HIGH, unfixed ignorés) ; environnement 'production' à créer dans les réglages GitHub avec relecteurs ; déploiement manuel lancé depuis main ; actions épinglées par SHA (checkout v4.2.2, etc.).</t>
-        </is>
-      </c>
-      <c r="H41" s="5" t="inlineStr">
-        <is>
-          <t>Premier run possiblement rouge (vulnérabilité de l'image de base, version d'action) : à corriger après le premier push.</t>
-        </is>
-      </c>
-      <c r="I41" s="5" t="inlineStr">
-        <is>
-          <t>en attente</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="C5:C41">
+  <conditionalFormatting sqref="C5:C18">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"NON_FAIT"</formula>
     </cfRule>
@@ -16700,7 +15627,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>VALIDEE</t>
+          <t>NON_DEMARREE</t>
         </is>
       </c>
     </row>
@@ -16722,8 +15649,9 @@
           <t>Avancement</t>
         </is>
       </c>
-      <c r="B5" s="12" t="n">
-        <v>1</v>
+      <c r="B5" s="12">
+        <f>IF(COUNTA(B8:B200)=0,0,(COUNTIF(F8:F200,"A_VALIDER")+COUNTIF(F8:F200,"VALIDE"))/COUNTA(B8:B200))</f>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -16811,17 +15739,17 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
+          <t>NON_FAIT</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Gprojet.slnx ; un seul projet backend src/Gprojet-Backend/Gprojet-Backend.csproj (Microsoft.NET.Sdk.Web, RootNamespace Gprojet.Backend) avec les dossiers-couches Web/, Orchestration/, Services/, Mapping/, Repositories/, Entities/, Contracts/, Infrastructure/, Common/ (espaces de noms alignés sur les dossiers) ; projet de tests tests/Gprojet-Backend.Tests (xUnit) avec Unitaires/, Integration/, Architecture/. Aucun autre projet (le front arrive en P2-T01). Demandes utilisateur à intégrer dans cette tâche : Directory.Packages.props → FluentAssertions en dernière 7.x stable (licence Apache 2.0, H-017) au lieu de 8.x ; migrer .gitlab/ vers .github/ (pull_request_template.md, ISSUE_TEMPLATE/Anomalie.md et Demande.md) et adapter CONTRIBUTING.md (pull requests GitHub).</t>
+          <t>Gprojet.slnx ; un seul projet backend src/Gprojet-Backend/Gprojet-Backend.csproj (Microsoft.NET.Sdk.Web, RootNamespace Gprojet.Backend) avec les dossiers-couches Web/, Orchestration/, Services/, Mapping/, Repositories/, Entities/, Contracts/, Infrastructure/, Common/ (espaces de noms alignés sur les dossiers) ; projet de tests tests/Gprojet-Backend.Tests (xUnit) avec Unitaires/, Integration/, Architecture/. Aucun autre projet (le front arrive en P2-T01).</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>dotnet build Gprojet.slnx réussit sans avertissement ; dotnet sln Gprojet.slnx list affiche exactement 2 projets (Gprojet-Backend, Gprojet-Backend.Tests) ; dotnet test passe (test de fumée). Directory.Packages.props référence FluentAssertions 7.x ; .gitlab/ n'existe plus et .github/pull_request_template.md existe.</t>
+          <t>dotnet build Gprojet.slnx réussit sans avertissement ; dotnet sln Gprojet.slnx list affiche exactement 2 projets (Gprojet-Backend, Gprojet-Backend.Tests) ; dotnet test passe (test de fumée).</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr"/>
@@ -16853,7 +15781,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
+          <t>NON_FAIT</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
@@ -16867,11 +15795,7 @@
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr"/>
-      <c r="J9" s="5" t="inlineStr">
-        <is>
-          <t>H-019 (OUVERTE)</t>
-        </is>
-      </c>
+      <c r="J9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
@@ -16899,7 +15823,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
+          <t>NON_FAIT</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
@@ -16913,11 +15837,7 @@
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr"/>
-      <c r="J10" s="5" t="inlineStr">
-        <is>
-          <t>H-020 (OUVERTE)</t>
-        </is>
-      </c>
+      <c r="J10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
@@ -16945,7 +15865,7 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
+          <t>NON_FAIT</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
@@ -16959,11 +15879,7 @@
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr"/>
-      <c r="J11" s="5" t="inlineStr">
-        <is>
-          <t>H-021 (OUVERTE)</t>
-        </is>
-      </c>
+      <c r="J11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
@@ -16991,7 +15907,7 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
+          <t>NON_FAIT</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
@@ -17005,11 +15921,7 @@
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr"/>
-      <c r="J12" s="5" t="inlineStr">
-        <is>
-          <t>H-022 (OUVERTE)</t>
-        </is>
-      </c>
+      <c r="J12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
@@ -17037,7 +15949,7 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
+          <t>NON_FAIT</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
@@ -17051,11 +15963,7 @@
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr"/>
-      <c r="J13" s="5" t="inlineStr">
-        <is>
-          <t>H-023 (OUVERTE)</t>
-        </is>
-      </c>
+      <c r="J13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
@@ -17083,7 +15991,7 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
+          <t>NON_FAIT</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -17097,11 +16005,7 @@
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr"/>
-      <c r="J14" s="5" t="inlineStr">
-        <is>
-          <t>H-024 (OUVERTE)</t>
-        </is>
-      </c>
+      <c r="J14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
@@ -17129,7 +16033,7 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
+          <t>NON_FAIT</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
@@ -17143,11 +16047,7 @@
         </is>
       </c>
       <c r="I15" s="5" t="inlineStr"/>
-      <c r="J15" s="5" t="inlineStr">
-        <is>
-          <t>H-025 (OUVERTE)</t>
-        </is>
-      </c>
+      <c r="J15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
@@ -17175,7 +16075,7 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
+          <t>NON_FAIT</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
@@ -17191,8 +16091,7 @@
       <c r="I16" s="5" t="inlineStr"/>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>H-004 (REPONDUE)
-H-026 (OUVERTE)</t>
+          <t>H-004 (REPONDUE)</t>
         </is>
       </c>
     </row>
@@ -17222,7 +16121,7 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
+          <t>NON_FAIT</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
@@ -17236,11 +16135,7 @@
         </is>
       </c>
       <c r="I17" s="5" t="inlineStr"/>
-      <c r="J17" s="5" t="inlineStr">
-        <is>
-          <t>H-027 (OUVERTE)</t>
-        </is>
-      </c>
+      <c r="J17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
@@ -17268,7 +16163,7 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
+          <t>NON_FAIT</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
@@ -17282,11 +16177,7 @@
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr"/>
-      <c r="J18" s="5" t="inlineStr">
-        <is>
-          <t>H-028 (OUVERTE)</t>
-        </is>
-      </c>
+      <c r="J18" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -17425,7 +16316,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>VALIDEE</t>
+          <t>NON_DEMARREE</t>
         </is>
       </c>
     </row>
@@ -17447,8 +16338,9 @@
           <t>Avancement</t>
         </is>
       </c>
-      <c r="B5" s="12" t="n">
-        <v>1</v>
+      <c r="B5" s="12">
+        <f>IF(COUNTA(B8:B200)=0,0,(COUNTIF(F8:F200,"A_VALIDER")+COUNTIF(F8:F200,"VALIDE"))/COUNTA(B8:B200))</f>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -17536,7 +16428,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
+          <t>NON_FAIT</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
@@ -17550,11 +16442,7 @@
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr"/>
-      <c r="J8" s="5" t="inlineStr">
-        <is>
-          <t>H-029 (OUVERTE)</t>
-        </is>
-      </c>
+      <c r="J8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
@@ -17582,7 +16470,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
+          <t>NON_FAIT</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
@@ -17598,8 +16486,7 @@
       <c r="I9" s="5" t="inlineStr"/>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>H-014 (REPONDUE)
-H-030 (OUVERTE)</t>
+          <t>H-014 (REPONDUE)</t>
         </is>
       </c>
     </row>
@@ -17629,7 +16516,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
+          <t>NON_FAIT</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
@@ -17643,11 +16530,7 @@
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr"/>
-      <c r="J10" s="5" t="inlineStr">
-        <is>
-          <t>H-031 (OUVERTE)</t>
-        </is>
-      </c>
+      <c r="J10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
@@ -17675,7 +16558,7 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
+          <t>NON_FAIT</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
@@ -17717,7 +16600,7 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
+          <t>NON_FAIT</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
@@ -17759,7 +16642,7 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
+          <t>NON_FAIT</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
@@ -17773,11 +16656,7 @@
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr"/>
-      <c r="J13" s="5" t="inlineStr">
-        <is>
-          <t>H-032 (OUVERTE)</t>
-        </is>
-      </c>
+      <c r="J13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
@@ -17805,7 +16684,7 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
+          <t>NON_FAIT</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -17819,11 +16698,7 @@
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr"/>
-      <c r="J14" s="5" t="inlineStr">
-        <is>
-          <t>H-033 (OUVERTE)</t>
-        </is>
-      </c>
+      <c r="J14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
@@ -17851,7 +16726,7 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
+          <t>NON_FAIT</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
@@ -17865,11 +16740,7 @@
         </is>
       </c>
       <c r="I15" s="5" t="inlineStr"/>
-      <c r="J15" s="5" t="inlineStr">
-        <is>
-          <t>H-034 (OUVERTE)</t>
-        </is>
-      </c>
+      <c r="J15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
@@ -17897,7 +16768,7 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
+          <t>NON_FAIT</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
@@ -17911,11 +16782,7 @@
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr"/>
-      <c r="J16" s="5" t="inlineStr">
-        <is>
-          <t>H-035 (OUVERTE)</t>
-        </is>
-      </c>
+      <c r="J16" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -18035,14 +16902,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>P3 · Conteneurisation et intégration continue GitHub Actions</t>
+          <t>P3 · Conteneurisation et intégration continue GitLab</t>
         </is>
       </c>
     </row>
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>Objectif : images Docker, environnement local complet par docker compose, intégration continue GitHub Actions sur le dépôt hajar-hamid-coder/gprojet. Livrable : docker compose up fonctionnel et .github/workflows/ci.yml. ⚠️ Nécessite Docker (hypothèse H-001).</t>
+          <t>Objectif : images Docker, environnement local complet par docker compose, pipeline GitLab CI. Livrable : docker compose up fonctionnel et .gitlab-ci.yml. ⚠️ Nécessite Docker (hypothèse H-001).</t>
         </is>
       </c>
     </row>
@@ -18054,7 +16921,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>VALIDEE</t>
+          <t>NON_DEMARREE</t>
         </is>
       </c>
     </row>
@@ -18076,8 +16943,9 @@
           <t>Avancement</t>
         </is>
       </c>
-      <c r="B5" s="12" t="n">
-        <v>1</v>
+      <c r="B5" s="12">
+        <f>IF(COUNTA(B8:B200)=0,0,(COUNTIF(F8:F200,"A_VALIDER")+COUNTIF(F8:F200,"VALIDE"))/COUNTA(B8:B200))</f>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -18165,7 +17033,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
+          <t>NON_FAIT</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
@@ -18211,7 +17079,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
+          <t>NON_FAIT</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
@@ -18225,11 +17093,7 @@
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr"/>
-      <c r="J9" s="5" t="inlineStr">
-        <is>
-          <t>H-036 (OUVERTE)</t>
-        </is>
-      </c>
+      <c r="J9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
@@ -18257,7 +17121,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
+          <t>NON_FAIT</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
@@ -18284,7 +17148,7 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Workflow GitHub Actions</t>
+          <t>Pipeline .gitlab-ci.yml</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -18299,24 +17163,23 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
+          <t>NON_FAIT</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>.github/workflows/ci.yml déclenché sur push et pull request : jobs build, test (service postgres:18, GP_TEST_CONNECTION, rapport de tests et couverture publiés comme artefacts), qualite (dotnet format --verify-no-changes), securite (CodeQL C#, dependency-review sur les pull requests, scan d'image Trivy), paquet (build et push de l'image vers GitHub Container Registry ghcr.io sur main et les tags, avec GITHUB_TOKEN), deploiement (workflow_dispatch + environnement protégé, préparé pour P13). Cache NuGet, versions d'actions épinglées. Vérifier que les modèles .github/ (faits en P1-T01) sont cohérents avec le workflow.</t>
+          <t>étapes build, test (service postgres:18, rapports JUnit et couverture Cobertura), qualite (dotnet format --verify-no-changes), securite (templates GitLab SAST, Dependency-Scanning, Secret-Detection, Container-Scanning), paquet (build et push des images vers le GitLab Container Registry sur main et les tags), deploiement (manuel, préparé pour P13). Cache NuGet.</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>python scripts/verifier-ci.py (à écrire, parse YAML) confirme les 6 jobs, leurs dépendances, le service PostgreSQL et l'absence de secret en clair ; les modèles .github/ sont présents. L'exécution réelle sur GitHub se constate après le push de l'utilisateur (signalé dans le bilan de phase).</t>
+          <t>python scripts/verifier-ci.py (à écrire, parse YAML) confirme les 6 étapes, les rapports JUnit, l'absence de secret en clair ; validation par l'API CI Lint de GitLab si H-002 est répondue, sinon signalée dans la preuve.</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr"/>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>H-002 (REPONDUE)
-H-037 (OUVERTE)</t>
+          <t>H-002 (OUVERTE)</t>
         </is>
       </c>
     </row>
@@ -18346,12 +17209,12 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>VALIDE</t>
+          <t>NON_FAIT</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>docs/DEPLOIEMENT.md : prérequis, variables, démarrage compose, migrations, dépannage, description du workflow GitHub Actions, des secrets à créer (Settings → Secrets and variables → Actions) et de la publication d'image sur ghcr.io.</t>
+          <t>docs/DEPLOIEMENT.md : prérequis, variables, démarrage compose, migrations, dépannage, description du pipeline et des variables CI à créer dans GitLab (masquées / protégées).</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
@@ -18521,8 +17384,9 @@
           <t>Avancement</t>
         </is>
       </c>
-      <c r="B5" s="12" t="n">
-        <v>0</v>
+      <c r="B5" s="12">
+        <f>IF(COUNTA(B8:B200)=0,0,(COUNTIF(F8:F200,"A_VALIDER")+COUNTIF(F8:F200,"VALIDE"))/COUNTA(B8:B200))</f>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -19079,8 +17943,9 @@
           <t>Avancement</t>
         </is>
       </c>
-      <c r="B5" s="12" t="n">
-        <v>0</v>
+      <c r="B5" s="12">
+        <f>IF(COUNTA(B8:B200)=0,0,(COUNTIF(F8:F200,"A_VALIDER")+COUNTIF(F8:F200,"VALIDE"))/COUNTA(B8:B200))</f>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -19721,8 +18586,9 @@
           <t>Avancement</t>
         </is>
       </c>
-      <c r="B5" s="12" t="n">
-        <v>0</v>
+      <c r="B5" s="12">
+        <f>IF(COUNTA(B8:B200)=0,0,(COUNTIF(F8:F200,"A_VALIDER")+COUNTIF(F8:F200,"VALIDE"))/COUNTA(B8:B200))</f>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -20451,8 +19317,9 @@
           <t>Avancement</t>
         </is>
       </c>
-      <c r="B5" s="12" t="n">
-        <v>0</v>
+      <c r="B5" s="12">
+        <f>IF(COUNTA(B8:B200)=0,0,(COUNTIF(F8:F200,"A_VALIDER")+COUNTIF(F8:F200,"VALIDE"))/COUNTA(B8:B200))</f>
+        <v/>
       </c>
     </row>
     <row r="6">

</xml_diff>